<commit_message>
Update budget 2027 with annualized 2026 figures and add IL Online row
P/Q (units/amount 2026) for Super Pharm, Life, and Salus now use the
annualized 2026 values instead of partial-year actuals; K/L/N/O
unchanged. Adds the previously-empty IL Online row (114 - IL online)
with all 6 fields filled. File stays at 4 sheets, no copied source
data.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-09-20-budget-2027.xlsx
+++ b/kirill/outputs/2026-09-20-budget-2027.xlsx
@@ -1071,14 +1071,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * \-??_ ;_ @_ "/>
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="0%"/>
     <numFmt numFmtId="168" formatCode="#,##0"/>
-    <numFmt numFmtId="169" formatCode="mmm\-yy"/>
-    <numFmt numFmtId="170" formatCode="General"/>
+    <numFmt numFmtId="169" formatCode="#,##0.00"/>
+    <numFmt numFmtId="170" formatCode="mmm\-yy"/>
+    <numFmt numFmtId="171" formatCode="General"/>
   </numFmts>
   <fonts count="25">
     <font>
@@ -1739,7 +1740,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="163">
+  <cellXfs count="164">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2132,6 +2133,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="169" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2236,7 +2241,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2244,7 +2249,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="42" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="42" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2252,11 +2257,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="44" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="44" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="45" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="45" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -10970,24 +10975,24 @@
       <c r="K3" s="97" t="n">
         <v>118392</v>
       </c>
-      <c r="L3" s="97" t="n">
+      <c r="L3" s="98" t="n">
         <v>1708656.85</v>
       </c>
       <c r="N3" s="97" t="n">
         <v>0</v>
       </c>
-      <c r="O3" s="97" t="n">
+      <c r="O3" s="98" t="n">
         <v>0</v>
       </c>
       <c r="P3" s="97" t="n">
-        <v>62455</v>
-      </c>
-      <c r="Q3" s="97" t="n">
-        <v>1113833.85</v>
+        <v>78890.5263157895</v>
+      </c>
+      <c r="Q3" s="98" t="n">
+        <v>1406948.02105263</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="98" t="n">
+      <c r="A4" s="99" t="n">
         <v>1</v>
       </c>
       <c r="B4" s="95" t="s">
@@ -11017,24 +11022,24 @@
       <c r="K4" s="97" t="n">
         <v>176505</v>
       </c>
-      <c r="L4" s="97" t="n">
+      <c r="L4" s="98" t="n">
         <v>6689220.5</v>
       </c>
       <c r="N4" s="97" t="n">
         <v>1952</v>
       </c>
-      <c r="O4" s="97" t="n">
+      <c r="O4" s="98" t="n">
         <v>147652.2</v>
       </c>
       <c r="P4" s="97" t="n">
-        <v>118307</v>
-      </c>
-      <c r="Q4" s="97" t="n">
-        <v>4476515.3</v>
+        <v>149440.421052632</v>
+      </c>
+      <c r="Q4" s="98" t="n">
+        <v>5654545.64210526</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="98" t="n">
+      <c r="A5" s="99" t="n">
         <v>7</v>
       </c>
       <c r="B5" s="95" t="s">
@@ -11061,15 +11066,15 @@
       <c r="I5" s="96" t="n">
         <v>1037274.565</v>
       </c>
-      <c r="K5" s="99"/>
-      <c r="L5" s="99"/>
-      <c r="N5" s="99"/>
-      <c r="O5" s="99"/>
-      <c r="P5" s="99"/>
-      <c r="Q5" s="99"/>
+      <c r="K5" s="100"/>
+      <c r="L5" s="100"/>
+      <c r="N5" s="100"/>
+      <c r="O5" s="100"/>
+      <c r="P5" s="100"/>
+      <c r="Q5" s="100"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="98" t="n">
+      <c r="A6" s="99" t="n">
         <v>4</v>
       </c>
       <c r="B6" s="95" t="s">
@@ -11096,15 +11101,15 @@
       <c r="I6" s="96" t="n">
         <v>2118523.978</v>
       </c>
-      <c r="K6" s="99"/>
-      <c r="L6" s="99"/>
-      <c r="N6" s="99"/>
-      <c r="O6" s="99"/>
-      <c r="P6" s="99"/>
-      <c r="Q6" s="99"/>
+      <c r="K6" s="100"/>
+      <c r="L6" s="100"/>
+      <c r="N6" s="100"/>
+      <c r="O6" s="100"/>
+      <c r="P6" s="100"/>
+      <c r="Q6" s="100"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="98" t="n">
+      <c r="A7" s="99" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="95" t="s">
@@ -11131,15 +11136,15 @@
       <c r="I7" s="96" t="n">
         <v>3722410.85</v>
       </c>
-      <c r="K7" s="99"/>
-      <c r="L7" s="99"/>
-      <c r="N7" s="99"/>
-      <c r="O7" s="99"/>
-      <c r="P7" s="99"/>
-      <c r="Q7" s="99"/>
+      <c r="K7" s="100"/>
+      <c r="L7" s="100"/>
+      <c r="N7" s="100"/>
+      <c r="O7" s="100"/>
+      <c r="P7" s="100"/>
+      <c r="Q7" s="100"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="98" t="n">
+      <c r="A8" s="99" t="n">
         <v>8</v>
       </c>
       <c r="B8" s="95" t="s">
@@ -11174,7 +11179,7 @@
       <c r="Q8" s="96"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="98" t="n">
+      <c r="A9" s="99" t="n">
         <v>6</v>
       </c>
       <c r="B9" s="95" t="s">
@@ -11201,15 +11206,15 @@
       <c r="I9" s="96" t="n">
         <v>1075277.57</v>
       </c>
-      <c r="K9" s="99"/>
-      <c r="L9" s="99"/>
-      <c r="N9" s="99"/>
-      <c r="O9" s="99"/>
-      <c r="P9" s="99"/>
-      <c r="Q9" s="99"/>
+      <c r="K9" s="100"/>
+      <c r="L9" s="100"/>
+      <c r="N9" s="100"/>
+      <c r="O9" s="100"/>
+      <c r="P9" s="100"/>
+      <c r="Q9" s="100"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="100" t="n">
+      <c r="A10" s="101" t="n">
         <v>10</v>
       </c>
       <c r="B10" s="95" t="s">
@@ -11236,15 +11241,15 @@
       <c r="I10" s="96" t="n">
         <v>151235.08</v>
       </c>
-      <c r="K10" s="99"/>
-      <c r="L10" s="99"/>
-      <c r="N10" s="99"/>
-      <c r="O10" s="99"/>
-      <c r="P10" s="99"/>
-      <c r="Q10" s="99"/>
+      <c r="K10" s="100"/>
+      <c r="L10" s="100"/>
+      <c r="N10" s="100"/>
+      <c r="O10" s="100"/>
+      <c r="P10" s="100"/>
+      <c r="Q10" s="100"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="98" t="n">
+      <c r="A11" s="99" t="n">
         <v>11</v>
       </c>
       <c r="B11" s="95" t="s">
@@ -11271,15 +11276,15 @@
       <c r="I11" s="96" t="n">
         <v>94015.41</v>
       </c>
-      <c r="K11" s="99"/>
-      <c r="L11" s="99"/>
-      <c r="N11" s="99"/>
-      <c r="O11" s="99"/>
-      <c r="P11" s="99"/>
-      <c r="Q11" s="99"/>
+      <c r="K11" s="100"/>
+      <c r="L11" s="100"/>
+      <c r="N11" s="100"/>
+      <c r="O11" s="100"/>
+      <c r="P11" s="100"/>
+      <c r="Q11" s="100"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="98" t="n">
+      <c r="A12" s="99" t="n">
         <v>14</v>
       </c>
       <c r="B12" s="95" t="s">
@@ -11306,15 +11311,15 @@
       <c r="I12" s="96" t="n">
         <v>33576.15</v>
       </c>
-      <c r="K12" s="99"/>
-      <c r="L12" s="99"/>
-      <c r="N12" s="99"/>
-      <c r="O12" s="99"/>
-      <c r="P12" s="99"/>
-      <c r="Q12" s="99"/>
+      <c r="K12" s="100"/>
+      <c r="L12" s="100"/>
+      <c r="N12" s="100"/>
+      <c r="O12" s="100"/>
+      <c r="P12" s="100"/>
+      <c r="Q12" s="100"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="98" t="n">
+      <c r="A13" s="99" t="n">
         <v>15</v>
       </c>
       <c r="B13" s="95" t="s">
@@ -11341,15 +11346,15 @@
       <c r="I13" s="96" t="n">
         <v>31896.82</v>
       </c>
-      <c r="K13" s="99"/>
-      <c r="L13" s="99"/>
-      <c r="N13" s="99"/>
-      <c r="O13" s="99"/>
-      <c r="P13" s="99"/>
-      <c r="Q13" s="99"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="100"/>
+      <c r="N13" s="100"/>
+      <c r="O13" s="100"/>
+      <c r="P13" s="100"/>
+      <c r="Q13" s="100"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="98" t="n">
+      <c r="A14" s="99" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="95" t="s">
@@ -11376,15 +11381,15 @@
       <c r="I14" s="96" t="n">
         <v>37748.72</v>
       </c>
-      <c r="K14" s="99"/>
-      <c r="L14" s="99"/>
-      <c r="N14" s="99"/>
-      <c r="O14" s="99"/>
-      <c r="P14" s="99"/>
-      <c r="Q14" s="99"/>
+      <c r="K14" s="100"/>
+      <c r="L14" s="100"/>
+      <c r="N14" s="100"/>
+      <c r="O14" s="100"/>
+      <c r="P14" s="100"/>
+      <c r="Q14" s="100"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="98" t="n">
+      <c r="A15" s="99" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="95" t="s">
@@ -11411,60 +11416,60 @@
       <c r="I15" s="96" t="n">
         <v>239111.1</v>
       </c>
-      <c r="K15" s="99"/>
-      <c r="L15" s="99"/>
-      <c r="N15" s="99"/>
-      <c r="O15" s="99"/>
-      <c r="P15" s="99"/>
-      <c r="Q15" s="99"/>
+      <c r="K15" s="100"/>
+      <c r="L15" s="100"/>
+      <c r="N15" s="100"/>
+      <c r="O15" s="100"/>
+      <c r="P15" s="100"/>
+      <c r="Q15" s="100"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102" t="s">
+      <c r="A16" s="102"/>
+      <c r="B16" s="103"/>
+      <c r="C16" s="103" t="s">
         <v>119</v>
       </c>
-      <c r="D16" s="102" t="s">
+      <c r="D16" s="103" t="s">
         <v>119</v>
       </c>
-      <c r="E16" s="102"/>
-      <c r="F16" s="102" t="n">
+      <c r="E16" s="103"/>
+      <c r="F16" s="103" t="n">
         <f aca="false">SUM(F3:F15)</f>
         <v>16644964.924</v>
       </c>
-      <c r="G16" s="102" t="n">
+      <c r="G16" s="103" t="n">
         <f aca="false">SUM(G3:G15)</f>
         <v>16462691.402</v>
       </c>
-      <c r="H16" s="102" t="n">
+      <c r="H16" s="103" t="n">
         <f aca="false">SUM(H3:H15)</f>
         <v>20641000</v>
       </c>
-      <c r="I16" s="102" t="n">
+      <c r="I16" s="103" t="n">
         <f aca="false">SUM(I3:I15)</f>
         <v>17499549.047</v>
       </c>
-      <c r="K16" s="102" t="n">
+      <c r="K16" s="103" t="n">
         <f aca="false">SUM(K3:K15)</f>
         <v>294897</v>
       </c>
-      <c r="L16" s="102" t="n">
+      <c r="L16" s="103" t="n">
         <f aca="false">SUM(L3:L15)</f>
         <v>8397877.35</v>
       </c>
-      <c r="N16" s="102" t="n">
+      <c r="N16" s="103" t="n">
         <f aca="false">SUM(N3:N15)</f>
         <v>1952</v>
       </c>
-      <c r="O16" s="102"/>
-      <c r="P16" s="102"/>
-      <c r="Q16" s="102" t="n">
+      <c r="O16" s="103"/>
+      <c r="P16" s="103"/>
+      <c r="Q16" s="103" t="n">
         <f aca="false">SUM(Q3:Q15)</f>
-        <v>5590349.15</v>
+        <v>7061493.66315789</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="98" t="n">
+      <c r="A17" s="99" t="n">
         <v>2</v>
       </c>
       <c r="B17" s="95" t="s">
@@ -11491,15 +11496,27 @@
       <c r="I17" s="96" t="n">
         <v>7612717.01355935</v>
       </c>
-      <c r="K17" s="99"/>
-      <c r="L17" s="99"/>
-      <c r="N17" s="99"/>
-      <c r="O17" s="99"/>
-      <c r="P17" s="99"/>
-      <c r="Q17" s="99"/>
+      <c r="K17" s="97" t="n">
+        <v>20470</v>
+      </c>
+      <c r="L17" s="98" t="n">
+        <v>1657320.76</v>
+      </c>
+      <c r="N17" s="97" t="n">
+        <v>2375</v>
+      </c>
+      <c r="O17" s="98" t="n">
+        <v>147591.2</v>
+      </c>
+      <c r="P17" s="97" t="n">
+        <v>36103.5789473684</v>
+      </c>
+      <c r="Q17" s="98" t="n">
+        <v>4037646.48</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="98" t="n">
+      <c r="A18" s="99" t="n">
         <v>12</v>
       </c>
       <c r="B18" s="95" t="s">
@@ -11526,60 +11543,60 @@
       <c r="I18" s="96" t="n">
         <v>39807.02</v>
       </c>
-      <c r="K18" s="99"/>
-      <c r="L18" s="99"/>
-      <c r="N18" s="99"/>
-      <c r="O18" s="99"/>
-      <c r="P18" s="99"/>
-      <c r="Q18" s="99"/>
+      <c r="K18" s="100"/>
+      <c r="L18" s="100"/>
+      <c r="N18" s="100"/>
+      <c r="O18" s="100"/>
+      <c r="P18" s="100"/>
+      <c r="Q18" s="100"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="100"/>
-      <c r="B19" s="102"/>
-      <c r="C19" s="102" t="s">
+      <c r="A19" s="101"/>
+      <c r="B19" s="103"/>
+      <c r="C19" s="103" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="102" t="s">
+      <c r="D19" s="103" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="102"/>
-      <c r="F19" s="102" t="n">
+      <c r="E19" s="103"/>
+      <c r="F19" s="103" t="n">
         <f aca="false">F16+F17+F18</f>
         <v>17364282.314</v>
       </c>
-      <c r="G19" s="102" t="n">
+      <c r="G19" s="103" t="n">
         <f aca="false">G16+G17+G18</f>
         <v>18146275.432</v>
       </c>
-      <c r="H19" s="102" t="n">
+      <c r="H19" s="103" t="n">
         <f aca="false">H16+H17+H18</f>
         <v>31460106.699322</v>
       </c>
-      <c r="I19" s="102" t="n">
+      <c r="I19" s="103" t="n">
         <f aca="false">I16+I17+I18</f>
         <v>25152073.0805594</v>
       </c>
-      <c r="K19" s="102" t="n">
+      <c r="K19" s="103" t="n">
         <f aca="false">K16+K17+K18</f>
-        <v>294897</v>
-      </c>
-      <c r="L19" s="102" t="n">
+        <v>315367</v>
+      </c>
+      <c r="L19" s="103" t="n">
         <f aca="false">L16+L17+L18</f>
-        <v>8397877.35</v>
-      </c>
-      <c r="N19" s="102" t="n">
+        <v>10055198.11</v>
+      </c>
+      <c r="N19" s="103" t="n">
         <f aca="false">N16+N17+N18</f>
-        <v>1952</v>
-      </c>
-      <c r="O19" s="102"/>
-      <c r="P19" s="102"/>
-      <c r="Q19" s="102" t="n">
+        <v>4327</v>
+      </c>
+      <c r="O19" s="103"/>
+      <c r="P19" s="103"/>
+      <c r="Q19" s="103" t="n">
         <f aca="false">Q16+Q17+Q18</f>
-        <v>5590349.15</v>
+        <v>11099140.1431579</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="100" t="n">
+      <c r="A20" s="101" t="n">
         <v>50</v>
       </c>
       <c r="B20" s="95" t="s">
@@ -11606,15 +11623,15 @@
       <c r="I20" s="96" t="n">
         <v>3098024.51</v>
       </c>
-      <c r="K20" s="99"/>
-      <c r="L20" s="99"/>
-      <c r="N20" s="99"/>
-      <c r="O20" s="99"/>
-      <c r="P20" s="99"/>
-      <c r="Q20" s="99"/>
+      <c r="K20" s="100"/>
+      <c r="L20" s="100"/>
+      <c r="N20" s="100"/>
+      <c r="O20" s="100"/>
+      <c r="P20" s="100"/>
+      <c r="Q20" s="100"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="100" t="n">
+      <c r="A21" s="101" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="95" t="s">
@@ -11641,15 +11658,15 @@
       <c r="I21" s="96" t="n">
         <v>922081.02</v>
       </c>
-      <c r="K21" s="99"/>
-      <c r="L21" s="99"/>
-      <c r="N21" s="99"/>
-      <c r="O21" s="99"/>
-      <c r="P21" s="99"/>
-      <c r="Q21" s="99"/>
+      <c r="K21" s="100"/>
+      <c r="L21" s="100"/>
+      <c r="N21" s="100"/>
+      <c r="O21" s="100"/>
+      <c r="P21" s="100"/>
+      <c r="Q21" s="100"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="100" t="n">
+      <c r="A22" s="101" t="n">
         <v>21</v>
       </c>
       <c r="B22" s="95" t="s">
@@ -11676,15 +11693,15 @@
       <c r="I22" s="96" t="n">
         <v>613276.52</v>
       </c>
-      <c r="K22" s="99"/>
-      <c r="L22" s="99"/>
-      <c r="N22" s="99"/>
-      <c r="O22" s="99"/>
-      <c r="P22" s="99"/>
-      <c r="Q22" s="99"/>
+      <c r="K22" s="100"/>
+      <c r="L22" s="100"/>
+      <c r="N22" s="100"/>
+      <c r="O22" s="100"/>
+      <c r="P22" s="100"/>
+      <c r="Q22" s="100"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="100" t="n">
+      <c r="A23" s="101" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="95" t="s">
@@ -11711,15 +11728,15 @@
       <c r="I23" s="96" t="n">
         <v>457053.13</v>
       </c>
-      <c r="K23" s="99"/>
-      <c r="L23" s="99"/>
-      <c r="N23" s="99"/>
-      <c r="O23" s="99"/>
-      <c r="P23" s="99"/>
-      <c r="Q23" s="99"/>
+      <c r="K23" s="100"/>
+      <c r="L23" s="100"/>
+      <c r="N23" s="100"/>
+      <c r="O23" s="100"/>
+      <c r="P23" s="100"/>
+      <c r="Q23" s="100"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="100" t="n">
+      <c r="A24" s="101" t="n">
         <v>23</v>
       </c>
       <c r="B24" s="95" t="s">
@@ -11746,15 +11763,15 @@
       <c r="I24" s="96" t="n">
         <v>131678.59</v>
       </c>
-      <c r="K24" s="99"/>
-      <c r="L24" s="99"/>
-      <c r="N24" s="99"/>
-      <c r="O24" s="99"/>
-      <c r="P24" s="99"/>
-      <c r="Q24" s="99"/>
+      <c r="K24" s="100"/>
+      <c r="L24" s="100"/>
+      <c r="N24" s="100"/>
+      <c r="O24" s="100"/>
+      <c r="P24" s="100"/>
+      <c r="Q24" s="100"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="100" t="n">
+      <c r="A25" s="101" t="n">
         <v>24</v>
       </c>
       <c r="B25" s="95" t="s">
@@ -11781,15 +11798,15 @@
       <c r="I25" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="99"/>
-      <c r="L25" s="99"/>
-      <c r="N25" s="99"/>
-      <c r="O25" s="99"/>
-      <c r="P25" s="99"/>
-      <c r="Q25" s="99"/>
+      <c r="K25" s="100"/>
+      <c r="L25" s="100"/>
+      <c r="N25" s="100"/>
+      <c r="O25" s="100"/>
+      <c r="P25" s="100"/>
+      <c r="Q25" s="100"/>
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="100" t="n">
+      <c r="A26" s="101" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="95" t="s">
@@ -11819,24 +11836,24 @@
       <c r="K26" s="97" t="n">
         <v>18268</v>
       </c>
-      <c r="L26" s="97" t="n">
+      <c r="L26" s="98" t="n">
         <v>319558.55</v>
       </c>
       <c r="N26" s="97" t="n">
         <v>991</v>
       </c>
-      <c r="O26" s="97" t="n">
+      <c r="O26" s="98" t="n">
         <v>14625</v>
       </c>
       <c r="P26" s="97" t="n">
-        <v>20601</v>
-      </c>
-      <c r="Q26" s="97" t="n">
-        <v>365555.25</v>
+        <v>26022.3157894737</v>
+      </c>
+      <c r="Q26" s="98" t="n">
+        <v>461754</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="100" t="n">
+      <c r="A27" s="101" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="95" t="s">
@@ -11863,15 +11880,15 @@
       <c r="I27" s="96" t="n">
         <v>100694.01</v>
       </c>
-      <c r="K27" s="99"/>
-      <c r="L27" s="99"/>
-      <c r="N27" s="99"/>
-      <c r="O27" s="99"/>
-      <c r="P27" s="99"/>
-      <c r="Q27" s="99"/>
+      <c r="K27" s="100"/>
+      <c r="L27" s="100"/>
+      <c r="N27" s="100"/>
+      <c r="O27" s="100"/>
+      <c r="P27" s="100"/>
+      <c r="Q27" s="100"/>
     </row>
     <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="100" t="n">
+      <c r="A28" s="101" t="n">
         <v>27</v>
       </c>
       <c r="B28" s="95" t="s">
@@ -11898,15 +11915,15 @@
       <c r="I28" s="96" t="n">
         <v>250000</v>
       </c>
-      <c r="K28" s="99"/>
-      <c r="L28" s="99"/>
-      <c r="N28" s="99"/>
-      <c r="O28" s="99"/>
-      <c r="P28" s="99"/>
-      <c r="Q28" s="99"/>
+      <c r="K28" s="100"/>
+      <c r="L28" s="100"/>
+      <c r="N28" s="100"/>
+      <c r="O28" s="100"/>
+      <c r="P28" s="100"/>
+      <c r="Q28" s="100"/>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="100" t="n">
+      <c r="A29" s="101" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="95" t="s">
@@ -11933,15 +11950,15 @@
       <c r="I29" s="96" t="n">
         <v>378207.09</v>
       </c>
-      <c r="K29" s="99"/>
-      <c r="L29" s="99"/>
-      <c r="N29" s="99"/>
-      <c r="O29" s="99"/>
-      <c r="P29" s="99"/>
-      <c r="Q29" s="99"/>
+      <c r="K29" s="100"/>
+      <c r="L29" s="100"/>
+      <c r="N29" s="100"/>
+      <c r="O29" s="100"/>
+      <c r="P29" s="100"/>
+      <c r="Q29" s="100"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="100" t="n">
+      <c r="A30" s="101" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="95" t="s">
@@ -11968,15 +11985,15 @@
       <c r="I30" s="96" t="n">
         <v>73116.44</v>
       </c>
-      <c r="K30" s="99"/>
-      <c r="L30" s="99"/>
-      <c r="N30" s="99"/>
-      <c r="O30" s="99"/>
-      <c r="P30" s="99"/>
-      <c r="Q30" s="99"/>
+      <c r="K30" s="100"/>
+      <c r="L30" s="100"/>
+      <c r="N30" s="100"/>
+      <c r="O30" s="100"/>
+      <c r="P30" s="100"/>
+      <c r="Q30" s="100"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="100" t="n">
+      <c r="A31" s="101" t="n">
         <v>30</v>
       </c>
       <c r="B31" s="95" t="s">
@@ -12003,15 +12020,15 @@
       <c r="I31" s="96" t="n">
         <v>42809.5</v>
       </c>
-      <c r="K31" s="99"/>
-      <c r="L31" s="99"/>
-      <c r="N31" s="99"/>
-      <c r="O31" s="99"/>
-      <c r="P31" s="99"/>
-      <c r="Q31" s="99"/>
+      <c r="K31" s="100"/>
+      <c r="L31" s="100"/>
+      <c r="N31" s="100"/>
+      <c r="O31" s="100"/>
+      <c r="P31" s="100"/>
+      <c r="Q31" s="100"/>
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="100" t="n">
+      <c r="A32" s="101" t="n">
         <v>31</v>
       </c>
       <c r="B32" s="95" t="s">
@@ -12038,15 +12055,15 @@
       <c r="I32" s="96" t="n">
         <v>17500</v>
       </c>
-      <c r="K32" s="99"/>
-      <c r="L32" s="99"/>
-      <c r="N32" s="99"/>
-      <c r="O32" s="99"/>
-      <c r="P32" s="99"/>
-      <c r="Q32" s="99"/>
+      <c r="K32" s="100"/>
+      <c r="L32" s="100"/>
+      <c r="N32" s="100"/>
+      <c r="O32" s="100"/>
+      <c r="P32" s="100"/>
+      <c r="Q32" s="100"/>
     </row>
     <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="100"/>
+      <c r="A33" s="101"/>
       <c r="B33" s="95"/>
       <c r="C33" s="95"/>
       <c r="D33" s="95" t="s">
@@ -12067,15 +12084,15 @@
       <c r="I33" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="K33" s="99"/>
-      <c r="L33" s="99"/>
-      <c r="N33" s="99"/>
-      <c r="O33" s="99"/>
-      <c r="P33" s="99"/>
-      <c r="Q33" s="99"/>
+      <c r="K33" s="100"/>
+      <c r="L33" s="100"/>
+      <c r="N33" s="100"/>
+      <c r="O33" s="100"/>
+      <c r="P33" s="100"/>
+      <c r="Q33" s="100"/>
     </row>
     <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="100" t="n">
+      <c r="A34" s="101" t="n">
         <v>32</v>
       </c>
       <c r="B34" s="95" t="s">
@@ -12102,15 +12119,15 @@
       <c r="I34" s="96" t="n">
         <v>38792.66</v>
       </c>
-      <c r="K34" s="99"/>
-      <c r="L34" s="99"/>
-      <c r="N34" s="99"/>
-      <c r="O34" s="99"/>
-      <c r="P34" s="99"/>
-      <c r="Q34" s="99"/>
+      <c r="K34" s="100"/>
+      <c r="L34" s="100"/>
+      <c r="N34" s="100"/>
+      <c r="O34" s="100"/>
+      <c r="P34" s="100"/>
+      <c r="Q34" s="100"/>
     </row>
     <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="100" t="n">
+      <c r="A35" s="101" t="n">
         <v>33</v>
       </c>
       <c r="B35" s="95" t="s">
@@ -12137,15 +12154,15 @@
       <c r="I35" s="96" t="n">
         <v>25000</v>
       </c>
-      <c r="K35" s="99"/>
-      <c r="L35" s="99"/>
-      <c r="N35" s="99"/>
-      <c r="O35" s="99"/>
-      <c r="P35" s="99"/>
-      <c r="Q35" s="99"/>
+      <c r="K35" s="100"/>
+      <c r="L35" s="100"/>
+      <c r="N35" s="100"/>
+      <c r="O35" s="100"/>
+      <c r="P35" s="100"/>
+      <c r="Q35" s="100"/>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="100"/>
+      <c r="A36" s="101"/>
       <c r="B36" s="95" t="s">
         <v>138</v>
       </c>
@@ -12170,15 +12187,15 @@
       <c r="I36" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="K36" s="99"/>
-      <c r="L36" s="99"/>
-      <c r="N36" s="99"/>
-      <c r="O36" s="99"/>
-      <c r="P36" s="99"/>
-      <c r="Q36" s="99"/>
+      <c r="K36" s="100"/>
+      <c r="L36" s="100"/>
+      <c r="N36" s="100"/>
+      <c r="O36" s="100"/>
+      <c r="P36" s="100"/>
+      <c r="Q36" s="100"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="100" t="n">
+      <c r="A37" s="101" t="n">
         <v>34</v>
       </c>
       <c r="B37" s="95" t="s">
@@ -12205,15 +12222,15 @@
       <c r="I37" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="K37" s="99"/>
-      <c r="L37" s="99"/>
-      <c r="N37" s="99"/>
-      <c r="O37" s="99"/>
-      <c r="P37" s="99"/>
-      <c r="Q37" s="99"/>
+      <c r="K37" s="100"/>
+      <c r="L37" s="100"/>
+      <c r="N37" s="100"/>
+      <c r="O37" s="100"/>
+      <c r="P37" s="100"/>
+      <c r="Q37" s="100"/>
     </row>
     <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="100" t="n">
+      <c r="A38" s="101" t="n">
         <v>35</v>
       </c>
       <c r="B38" s="95" t="s">
@@ -12240,15 +12257,15 @@
       <c r="I38" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="K38" s="99"/>
-      <c r="L38" s="99"/>
-      <c r="N38" s="99"/>
-      <c r="O38" s="99"/>
-      <c r="P38" s="99"/>
-      <c r="Q38" s="99"/>
+      <c r="K38" s="100"/>
+      <c r="L38" s="100"/>
+      <c r="N38" s="100"/>
+      <c r="O38" s="100"/>
+      <c r="P38" s="100"/>
+      <c r="Q38" s="100"/>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="100" t="n">
+      <c r="A39" s="101" t="n">
         <v>36</v>
       </c>
       <c r="B39" s="95"/>
@@ -12279,7 +12296,7 @@
       <c r="Q39" s="96"/>
     </row>
     <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="100" t="n">
+      <c r="A40" s="101" t="n">
         <v>37</v>
       </c>
       <c r="B40" s="95"/>
@@ -12300,7 +12317,7 @@
       <c r="Q40" s="96"/>
     </row>
     <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="100" t="n">
+      <c r="A41" s="101" t="n">
         <v>38</v>
       </c>
       <c r="B41" s="95"/>
@@ -12327,137 +12344,137 @@
       <c r="Q41" s="96"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="100"/>
-      <c r="B42" s="103"/>
-      <c r="C42" s="103" t="s">
+      <c r="A42" s="101"/>
+      <c r="B42" s="104"/>
+      <c r="C42" s="104" t="s">
         <v>98</v>
       </c>
-      <c r="D42" s="103" t="s">
+      <c r="D42" s="104" t="s">
         <v>98</v>
       </c>
-      <c r="E42" s="103"/>
-      <c r="F42" s="103" t="n">
+      <c r="E42" s="104"/>
+      <c r="F42" s="104" t="n">
         <f aca="false">SUM(F20:F41)</f>
         <v>7648509.62</v>
       </c>
-      <c r="G42" s="103" t="n">
+      <c r="G42" s="104" t="n">
         <f aca="false">SUM(G20:G41)</f>
         <v>5973375.8</v>
       </c>
-      <c r="H42" s="103" t="n">
+      <c r="H42" s="104" t="n">
         <f aca="false">SUM(H20:H41)</f>
         <v>9781372.5132875</v>
       </c>
-      <c r="I42" s="103" t="n">
+      <c r="I42" s="104" t="n">
         <f aca="false">SUM(I20:I41)</f>
         <v>6772380.94</v>
       </c>
-      <c r="K42" s="103" t="n">
+      <c r="K42" s="104" t="n">
         <f aca="false">SUM(K20:K41)</f>
         <v>18268</v>
       </c>
-      <c r="L42" s="103" t="n">
+      <c r="L42" s="104" t="n">
         <f aca="false">SUM(L20:L41)</f>
         <v>319558.55</v>
       </c>
-      <c r="N42" s="103" t="n">
+      <c r="N42" s="104" t="n">
         <f aca="false">SUM(N20:N41)</f>
         <v>991</v>
       </c>
-      <c r="O42" s="103"/>
-      <c r="P42" s="103"/>
-      <c r="Q42" s="103" t="n">
+      <c r="O42" s="104"/>
+      <c r="P42" s="104"/>
+      <c r="Q42" s="104" t="n">
         <f aca="false">SUM(Q20:Q41)</f>
-        <v>365555.25</v>
+        <v>461754</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="100"/>
-      <c r="B43" s="104"/>
-      <c r="C43" s="104" t="s">
+      <c r="A43" s="101"/>
+      <c r="B43" s="105"/>
+      <c r="C43" s="105" t="s">
         <v>144</v>
       </c>
-      <c r="D43" s="104" t="s">
+      <c r="D43" s="105" t="s">
         <v>144</v>
       </c>
-      <c r="E43" s="104"/>
-      <c r="F43" s="104" t="n">
+      <c r="E43" s="105"/>
+      <c r="F43" s="105" t="n">
         <f aca="false">F42+F19</f>
         <v>25012791.934</v>
       </c>
-      <c r="G43" s="104" t="n">
+      <c r="G43" s="105" t="n">
         <f aca="false">G42+G19</f>
         <v>24119651.232</v>
       </c>
-      <c r="H43" s="104" t="n">
+      <c r="H43" s="105" t="n">
         <f aca="false">H42+H19</f>
         <v>41241479.2126095</v>
       </c>
-      <c r="I43" s="104" t="n">
+      <c r="I43" s="105" t="n">
         <f aca="false">I42+I19</f>
         <v>31924454.0205594</v>
       </c>
-      <c r="K43" s="104" t="n">
+      <c r="K43" s="105" t="n">
         <f aca="false">K42+K19</f>
-        <v>313165</v>
-      </c>
-      <c r="L43" s="104" t="n">
+        <v>333635</v>
+      </c>
+      <c r="L43" s="105" t="n">
         <f aca="false">L42+L19</f>
-        <v>8717435.9</v>
-      </c>
-      <c r="N43" s="104" t="n">
+        <v>10374756.66</v>
+      </c>
+      <c r="N43" s="105" t="n">
         <f aca="false">N42+N19</f>
-        <v>2943</v>
-      </c>
-      <c r="O43" s="104"/>
-      <c r="P43" s="104"/>
-      <c r="Q43" s="104" t="n">
+        <v>5318</v>
+      </c>
+      <c r="O43" s="105"/>
+      <c r="P43" s="105"/>
+      <c r="Q43" s="105" t="n">
         <f aca="false">Q42+Q19</f>
-        <v>5955904.4</v>
+        <v>11560894.1431579</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="105"/>
-      <c r="C44" s="105" t="s">
+      <c r="B44" s="106"/>
+      <c r="C44" s="106" t="s">
         <v>145</v>
       </c>
-      <c r="D44" s="105" t="s">
+      <c r="D44" s="106" t="s">
         <v>145</v>
       </c>
-      <c r="E44" s="105"/>
-      <c r="F44" s="106" t="n">
+      <c r="E44" s="106"/>
+      <c r="F44" s="107" t="n">
         <f aca="false">F42/F43</f>
         <v>0.305783922090015</v>
       </c>
-      <c r="G44" s="106" t="n">
+      <c r="G44" s="107" t="n">
         <f aca="false">G42/G43</f>
         <v>0.247655977383081</v>
       </c>
-      <c r="H44" s="106" t="n">
+      <c r="H44" s="107" t="n">
         <f aca="false">H42/H43</f>
         <v>0.237173173708495</v>
       </c>
-      <c r="I44" s="106" t="n">
+      <c r="I44" s="107" t="n">
         <f aca="false">I42/I43</f>
         <v>0.212137721623636</v>
       </c>
-      <c r="K44" s="106" t="n">
+      <c r="K44" s="107" t="n">
         <f aca="false">IFERROR(K42/K43,"")</f>
-        <v>0.0583334663835358</v>
-      </c>
-      <c r="L44" s="106" t="n">
+        <v>0.0547544472252611</v>
+      </c>
+      <c r="L44" s="107" t="n">
         <f aca="false">IFERROR(L42/L43,"")</f>
-        <v>0.0366574017481448</v>
-      </c>
-      <c r="N44" s="106" t="n">
+        <v>0.0308015465299598</v>
+      </c>
+      <c r="N44" s="107" t="n">
         <f aca="false">IFERROR(N42/N43,"")</f>
-        <v>0.336731226639484</v>
-      </c>
-      <c r="O44" s="106"/>
-      <c r="P44" s="106"/>
-      <c r="Q44" s="106" t="n">
+        <v>0.186348251222264</v>
+      </c>
+      <c r="O44" s="107"/>
+      <c r="P44" s="107"/>
+      <c r="Q44" s="107" t="n">
         <f aca="false">IFERROR(Q42/Q43,"")</f>
-        <v>0.061376950576977</v>
+        <v>0.0399410282874427</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12480,159 +12497,159 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D47" s="102" t="s">
+      <c r="D47" s="103" t="s">
         <v>146</v>
       </c>
       <c r="E47" s="5"/>
-      <c r="F47" s="107" t="n">
+      <c r="F47" s="108" t="n">
         <f aca="false">F16</f>
         <v>16644964.924</v>
       </c>
-      <c r="G47" s="107" t="n">
+      <c r="G47" s="108" t="n">
         <f aca="false">G16</f>
         <v>16462691.402</v>
       </c>
-      <c r="H47" s="107" t="n">
+      <c r="H47" s="108" t="n">
         <f aca="false">H16</f>
         <v>20641000</v>
       </c>
-      <c r="I47" s="107" t="n">
+      <c r="I47" s="108" t="n">
         <f aca="false">I16</f>
         <v>17499549.047</v>
       </c>
-      <c r="K47" s="107" t="n">
+      <c r="K47" s="108" t="n">
         <f aca="false">K16</f>
         <v>294897</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D48" s="102" t="s">
+      <c r="D48" s="103" t="s">
         <v>147</v>
       </c>
       <c r="E48" s="5"/>
-      <c r="F48" s="107" t="n">
+      <c r="F48" s="108" t="n">
         <f aca="false">F17+F18</f>
         <v>719317.39</v>
       </c>
-      <c r="G48" s="107" t="n">
+      <c r="G48" s="108" t="n">
         <f aca="false">G17+G18</f>
         <v>1683584.03</v>
       </c>
-      <c r="H48" s="107" t="n">
+      <c r="H48" s="108" t="n">
         <f aca="false">H17+H18</f>
         <v>10819106.699322</v>
       </c>
-      <c r="I48" s="107" t="n">
+      <c r="I48" s="108" t="n">
         <f aca="false">I17+I18</f>
         <v>7652524.03355935</v>
       </c>
-      <c r="K48" s="107" t="n">
+      <c r="K48" s="108" t="n">
         <f aca="false">K17+K18</f>
-        <v>0</v>
+        <v>20470</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D49" s="108" t="s">
+      <c r="D49" s="109" t="s">
         <v>148</v>
       </c>
       <c r="E49" s="5"/>
-      <c r="F49" s="109" t="n">
+      <c r="F49" s="110" t="n">
         <f aca="false">SUM(F47:F48)</f>
         <v>17364282.314</v>
       </c>
-      <c r="G49" s="109" t="n">
+      <c r="G49" s="110" t="n">
         <f aca="false">SUM(G47:G48)</f>
         <v>18146275.432</v>
       </c>
-      <c r="H49" s="109" t="n">
+      <c r="H49" s="110" t="n">
         <f aca="false">SUM(H47:H48)</f>
         <v>31460106.699322</v>
       </c>
-      <c r="I49" s="109" t="n">
+      <c r="I49" s="110" t="n">
         <f aca="false">SUM(I47:I48)</f>
         <v>25152073.0805594</v>
       </c>
-      <c r="K49" s="109" t="n">
+      <c r="K49" s="110" t="n">
         <f aca="false">SUM(K47:K48)</f>
-        <v>294897</v>
+        <v>315367</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D51" s="102" t="s">
+      <c r="D51" s="103" t="s">
         <v>149</v>
       </c>
       <c r="E51" s="5"/>
-      <c r="F51" s="107" t="n">
+      <c r="F51" s="108" t="n">
         <f aca="false">F20</f>
         <v>3501494.53</v>
       </c>
-      <c r="G51" s="107" t="n">
+      <c r="G51" s="108" t="n">
         <f aca="false">G20</f>
         <v>2705391.22</v>
       </c>
-      <c r="H51" s="107" t="n">
+      <c r="H51" s="108" t="n">
         <f aca="false">H20</f>
         <v>4776579.3532875</v>
       </c>
-      <c r="I51" s="107" t="n">
+      <c r="I51" s="108" t="n">
         <f aca="false">I20</f>
         <v>3098024.51</v>
       </c>
-      <c r="K51" s="107" t="n">
+      <c r="K51" s="108" t="n">
         <f aca="false">K20</f>
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D52" s="102" t="s">
+      <c r="D52" s="103" t="s">
         <v>150</v>
       </c>
       <c r="E52" s="5"/>
-      <c r="F52" s="107" t="n">
+      <c r="F52" s="108" t="n">
         <f aca="false">SUM(F21:F41)</f>
         <v>4147015.09</v>
       </c>
-      <c r="G52" s="107" t="n">
+      <c r="G52" s="108" t="n">
         <f aca="false">SUM(G21:G41)</f>
         <v>3267984.58</v>
       </c>
-      <c r="H52" s="107" t="n">
+      <c r="H52" s="108" t="n">
         <f aca="false">SUM(H21:H41)</f>
         <v>5004793.16</v>
       </c>
-      <c r="I52" s="107" t="n">
+      <c r="I52" s="108" t="n">
         <f aca="false">SUM(I21:I41)</f>
         <v>3674356.43</v>
       </c>
-      <c r="K52" s="107" t="n">
+      <c r="K52" s="108" t="n">
         <f aca="false">SUM(K21:K41)</f>
         <v>18268</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D53" s="104" t="s">
+      <c r="D53" s="105" t="s">
         <v>151</v>
       </c>
       <c r="E53" s="5"/>
-      <c r="F53" s="104" t="n">
+      <c r="F53" s="105" t="n">
         <f aca="false">SUM(F49:F52)</f>
         <v>25012791.934</v>
       </c>
-      <c r="G53" s="104" t="n">
+      <c r="G53" s="105" t="n">
         <f aca="false">SUM(G49:G52)</f>
         <v>24119651.232</v>
       </c>
-      <c r="H53" s="104" t="n">
+      <c r="H53" s="105" t="n">
         <f aca="false">SUM(H49:H52)</f>
         <v>41241479.2126095</v>
       </c>
-      <c r="I53" s="104" t="n">
+      <c r="I53" s="105" t="n">
         <f aca="false">SUM(I49:I52)</f>
         <v>31924454.0205594</v>
       </c>
-      <c r="K53" s="104" t="n">
+      <c r="K53" s="105" t="n">
         <f aca="false">SUM(K49:K52)</f>
-        <v>313165</v>
+        <v>333635</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12660,84 +12677,84 @@
   <dimension ref="A1:AD78"/>
   <sheetFormatPr defaultColWidth="8.6171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="110" width="19.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="110" width="14.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="110" width="9.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="111" width="19.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="111" width="14.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="111" width="9.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="8.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="111" width="15.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="112" width="15.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="5" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="112" t="s">
+      <c r="C1" s="113" t="s">
         <v>153</v>
       </c>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="J1" s="113" t="s">
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
+      <c r="H1" s="113"/>
+      <c r="J1" s="114" t="s">
         <v>102</v>
       </c>
-      <c r="K1" s="113"/>
-      <c r="L1" s="113"/>
-    </row>
-    <row r="2" s="115" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="114" t="s">
+      <c r="K1" s="114"/>
+      <c r="L1" s="114"/>
+    </row>
+    <row r="2" s="116" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="115" t="s">
         <v>154</v>
       </c>
-      <c r="B2" s="110" t="s">
+      <c r="B2" s="111" t="s">
         <v>155</v>
       </c>
-      <c r="C2" s="110" t="s">
+      <c r="C2" s="111" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="110" t="s">
+      <c r="D2" s="111" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="110" t="s">
+      <c r="E2" s="111" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="115" t="s">
+      <c r="F2" s="116" t="s">
         <v>156</v>
       </c>
-      <c r="G2" s="115" t="s">
+      <c r="G2" s="116" t="s">
         <v>157</v>
       </c>
-      <c r="H2" s="115" t="s">
+      <c r="H2" s="116" t="s">
         <v>158</v>
       </c>
-      <c r="J2" s="115" t="s">
+      <c r="J2" s="116" t="s">
         <v>159</v>
       </c>
-      <c r="K2" s="115" t="s">
+      <c r="K2" s="116" t="s">
         <v>157</v>
       </c>
-      <c r="L2" s="115" t="s">
+      <c r="L2" s="116" t="s">
         <v>158</v>
       </c>
-      <c r="M2" s="115" t="s">
+      <c r="M2" s="116" t="s">
         <v>160</v>
       </c>
-      <c r="N2" s="116" t="s">
+      <c r="N2" s="117" t="s">
         <v>161</v>
       </c>
-      <c r="O2" s="117" t="s">
+      <c r="O2" s="118" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="110" t="s">
+      <c r="A3" s="111" t="s">
         <v>163</v>
       </c>
-      <c r="B3" s="110" t="n">
+      <c r="B3" s="111" t="n">
         <v>2025</v>
       </c>
       <c r="C3" s="5" t="n">
@@ -12781,7 +12798,7 @@
       <c r="M3" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="N3" s="118" t="s">
+      <c r="N3" s="119" t="s">
         <v>165</v>
       </c>
       <c r="O3" s="5" t="n">
@@ -12790,10 +12807,10 @@
       <c r="P3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="110" t="s">
+      <c r="A4" s="111" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="110" t="n">
+      <c r="B4" s="111" t="n">
         <v>2025</v>
       </c>
       <c r="C4" s="5" t="n">
@@ -12836,7 +12853,7 @@
       <c r="M4" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="N4" s="118" t="s">
+      <c r="N4" s="119" t="s">
         <v>167</v>
       </c>
       <c r="O4" s="5" t="n">
@@ -12844,10 +12861,10 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="119" t="s">
+      <c r="A5" s="120" t="s">
         <v>168</v>
       </c>
-      <c r="B5" s="110" t="n">
+      <c r="B5" s="111" t="n">
         <v>2025</v>
       </c>
       <c r="D5" s="5" t="n">
@@ -12867,7 +12884,7 @@
       <c r="I5" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="J5" s="120" t="n">
+      <c r="J5" s="121" t="n">
         <v>2000</v>
       </c>
       <c r="K5" s="5" t="n">
@@ -12881,55 +12898,55 @@
       <c r="M5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="N5" s="118" t="s">
+      <c r="N5" s="119" t="s">
         <v>169</v>
       </c>
-      <c r="P5" s="121" t="s">
+      <c r="P5" s="122" t="s">
         <v>170</v>
       </c>
-      <c r="Q5" s="122" t="s">
+      <c r="Q5" s="123" t="s">
         <v>4</v>
       </c>
-      <c r="R5" s="122" t="s">
+      <c r="R5" s="123" t="s">
         <v>5</v>
       </c>
-      <c r="S5" s="122" t="s">
+      <c r="S5" s="123" t="s">
         <v>6</v>
       </c>
-      <c r="T5" s="122" t="s">
+      <c r="T5" s="123" t="s">
         <v>7</v>
       </c>
-      <c r="U5" s="122" t="s">
+      <c r="U5" s="123" t="s">
         <v>8</v>
       </c>
-      <c r="V5" s="122" t="s">
+      <c r="V5" s="123" t="s">
         <v>9</v>
       </c>
-      <c r="W5" s="122" t="s">
+      <c r="W5" s="123" t="s">
         <v>10</v>
       </c>
-      <c r="X5" s="122" t="s">
+      <c r="X5" s="123" t="s">
         <v>11</v>
       </c>
-      <c r="Y5" s="122" t="s">
+      <c r="Y5" s="123" t="s">
         <v>12</v>
       </c>
-      <c r="Z5" s="122" t="s">
+      <c r="Z5" s="123" t="s">
         <v>13</v>
       </c>
-      <c r="AA5" s="122" t="s">
+      <c r="AA5" s="123" t="s">
         <v>14</v>
       </c>
-      <c r="AB5" s="122" t="s">
+      <c r="AB5" s="123" t="s">
         <v>15</v>
       </c>
-      <c r="AC5" s="123"/>
+      <c r="AC5" s="124"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="110" t="s">
+      <c r="A6" s="111" t="s">
         <v>170</v>
       </c>
-      <c r="B6" s="124" t="n">
+      <c r="B6" s="125" t="n">
         <v>46023</v>
       </c>
       <c r="F6" s="5" t="n">
@@ -12946,7 +12963,7 @@
       <c r="I6" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="J6" s="120" t="n">
+      <c r="J6" s="121" t="n">
         <v>1000</v>
       </c>
       <c r="K6" s="5" t="n">
@@ -12960,13 +12977,13 @@
       <c r="M6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="N6" s="118" t="s">
+      <c r="N6" s="119" t="s">
         <v>171</v>
       </c>
       <c r="O6" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="P6" s="125" t="s">
+      <c r="P6" s="126" t="s">
         <v>172</v>
       </c>
       <c r="Q6" s="1" t="n">
@@ -13005,16 +13022,16 @@
       <c r="AB6" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AC6" s="126" t="n">
+      <c r="AC6" s="127" t="n">
         <f aca="false">SUM(Q6:AB6)</f>
         <v>300</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="110" t="s">
+      <c r="A7" s="111" t="s">
         <v>173</v>
       </c>
-      <c r="B7" s="124" t="n">
+      <c r="B7" s="125" t="n">
         <v>46023</v>
       </c>
       <c r="F7" s="5" t="n">
@@ -13045,13 +13062,13 @@
       <c r="M7" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="N7" s="118" t="s">
+      <c r="N7" s="119" t="s">
         <v>171</v>
       </c>
       <c r="O7" s="5" t="n">
         <v>220</v>
       </c>
-      <c r="P7" s="125" t="s">
+      <c r="P7" s="126" t="s">
         <v>174</v>
       </c>
       <c r="Q7" s="1" t="n">
@@ -13090,16 +13107,16 @@
       <c r="AB7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="AC7" s="126"/>
+      <c r="AC7" s="127"/>
       <c r="AD7" s="1" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="110" t="s">
+      <c r="A8" s="111" t="s">
         <v>176</v>
       </c>
-      <c r="B8" s="110" t="s">
+      <c r="B8" s="111" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="5"/>
@@ -13128,56 +13145,56 @@
       <c r="M8" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="P8" s="127"/>
-      <c r="Q8" s="128" t="n">
+      <c r="P8" s="128"/>
+      <c r="Q8" s="129" t="n">
         <f aca="false">Q6*2</f>
         <v>140</v>
       </c>
-      <c r="R8" s="128" t="n">
+      <c r="R8" s="129" t="n">
         <f aca="false">R6*2</f>
         <v>40</v>
       </c>
-      <c r="S8" s="128" t="n">
+      <c r="S8" s="129" t="n">
         <f aca="false">S6*2</f>
         <v>60</v>
       </c>
-      <c r="T8" s="128" t="n">
+      <c r="T8" s="129" t="n">
         <f aca="false">T6*2</f>
         <v>40</v>
       </c>
-      <c r="U8" s="128" t="n">
+      <c r="U8" s="129" t="n">
         <f aca="false">U6*2</f>
         <v>40</v>
       </c>
-      <c r="V8" s="128" t="n">
+      <c r="V8" s="129" t="n">
         <f aca="false">V6*2</f>
         <v>60</v>
       </c>
-      <c r="W8" s="128" t="n">
+      <c r="W8" s="129" t="n">
         <f aca="false">W6*2</f>
         <v>50</v>
       </c>
-      <c r="X8" s="128" t="n">
+      <c r="X8" s="129" t="n">
         <f aca="false">X6*2</f>
         <v>50</v>
       </c>
-      <c r="Y8" s="128" t="n">
+      <c r="Y8" s="129" t="n">
         <f aca="false">Y6*2</f>
         <v>20</v>
       </c>
-      <c r="Z8" s="128" t="n">
+      <c r="Z8" s="129" t="n">
         <f aca="false">Z6*2</f>
         <v>20</v>
       </c>
-      <c r="AA8" s="128" t="n">
+      <c r="AA8" s="129" t="n">
         <f aca="false">AA6*2</f>
         <v>60</v>
       </c>
-      <c r="AB8" s="128" t="n">
+      <c r="AB8" s="129" t="n">
         <f aca="false">AB6*2</f>
         <v>20</v>
       </c>
-      <c r="AC8" s="129" t="n">
+      <c r="AC8" s="130" t="n">
         <f aca="false">SUM(Q8:AB8)</f>
         <v>600</v>
       </c>
@@ -13186,10 +13203,10 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="110" t="s">
+      <c r="A9" s="111" t="s">
         <v>177</v>
       </c>
-      <c r="B9" s="110" t="s">
+      <c r="B9" s="111" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="5"/>
@@ -13217,10 +13234,10 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="110" t="s">
+      <c r="A10" s="111" t="s">
         <v>178</v>
       </c>
-      <c r="B10" s="110" t="s">
+      <c r="B10" s="111" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="5"/>
@@ -13245,52 +13262,52 @@
       <c r="M10" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="P10" s="121" t="s">
+      <c r="P10" s="122" t="s">
         <v>179</v>
       </c>
-      <c r="Q10" s="122" t="s">
+      <c r="Q10" s="123" t="s">
         <v>4</v>
       </c>
-      <c r="R10" s="122" t="s">
+      <c r="R10" s="123" t="s">
         <v>5</v>
       </c>
-      <c r="S10" s="122" t="s">
+      <c r="S10" s="123" t="s">
         <v>6</v>
       </c>
-      <c r="T10" s="122" t="s">
+      <c r="T10" s="123" t="s">
         <v>7</v>
       </c>
-      <c r="U10" s="122" t="s">
+      <c r="U10" s="123" t="s">
         <v>8</v>
       </c>
-      <c r="V10" s="122" t="s">
+      <c r="V10" s="123" t="s">
         <v>9</v>
       </c>
-      <c r="W10" s="122" t="s">
+      <c r="W10" s="123" t="s">
         <v>10</v>
       </c>
-      <c r="X10" s="122" t="s">
+      <c r="X10" s="123" t="s">
         <v>11</v>
       </c>
-      <c r="Y10" s="122" t="s">
+      <c r="Y10" s="123" t="s">
         <v>12</v>
       </c>
-      <c r="Z10" s="122" t="s">
+      <c r="Z10" s="123" t="s">
         <v>13</v>
       </c>
-      <c r="AA10" s="122" t="s">
+      <c r="AA10" s="123" t="s">
         <v>14</v>
       </c>
-      <c r="AB10" s="122" t="s">
+      <c r="AB10" s="123" t="s">
         <v>15</v>
       </c>
-      <c r="AC10" s="123"/>
+      <c r="AC10" s="124"/>
       <c r="AD10" s="1" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="110" t="s">
+      <c r="A11" s="111" t="s">
         <v>181</v>
       </c>
       <c r="B11" s="5" t="s">
@@ -13318,13 +13335,13 @@
       <c r="M11" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="N11" s="118" t="s">
+      <c r="N11" s="119" t="s">
         <v>182</v>
       </c>
       <c r="O11" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="P11" s="125" t="s">
+      <c r="P11" s="126" t="s">
         <v>172</v>
       </c>
       <c r="V11" s="1" t="n">
@@ -13348,13 +13365,13 @@
       <c r="AB11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AC11" s="126" t="n">
+      <c r="AC11" s="127" t="n">
         <f aca="false">SUM(Q11:AB11)</f>
         <v>140</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="110" t="s">
+      <c r="A12" s="111" t="s">
         <v>183</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -13367,7 +13384,7 @@
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
-      <c r="J12" s="120"/>
+      <c r="J12" s="121"/>
       <c r="K12" s="5" t="n">
         <v>130</v>
       </c>
@@ -13378,8 +13395,8 @@
       <c r="M12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="N12" s="118"/>
-      <c r="P12" s="125" t="s">
+      <c r="N12" s="119"/>
+      <c r="P12" s="126" t="s">
         <v>174</v>
       </c>
       <c r="V12" s="1" t="n">
@@ -13403,10 +13420,10 @@
       <c r="AB12" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="AC12" s="126"/>
+      <c r="AC12" s="127"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="110" t="s">
+      <c r="A13" s="111" t="s">
         <v>184</v>
       </c>
       <c r="B13" s="5"/>
@@ -13432,71 +13449,71 @@
       <c r="M13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="N13" s="118" t="s">
+      <c r="N13" s="119" t="s">
         <v>185</v>
       </c>
       <c r="O13" s="5" t="n">
         <v>2016</v>
       </c>
-      <c r="P13" s="127"/>
-      <c r="Q13" s="128" t="n">
+      <c r="P13" s="128"/>
+      <c r="Q13" s="129" t="n">
         <f aca="false">Q11*2</f>
         <v>0</v>
       </c>
-      <c r="R13" s="128" t="n">
+      <c r="R13" s="129" t="n">
         <f aca="false">R11*2</f>
         <v>0</v>
       </c>
-      <c r="S13" s="128" t="n">
+      <c r="S13" s="129" t="n">
         <f aca="false">S11*2</f>
         <v>0</v>
       </c>
-      <c r="T13" s="128" t="n">
+      <c r="T13" s="129" t="n">
         <f aca="false">T11*2</f>
         <v>0</v>
       </c>
-      <c r="U13" s="128" t="n">
+      <c r="U13" s="129" t="n">
         <f aca="false">U11*2</f>
         <v>0</v>
       </c>
-      <c r="V13" s="128" t="n">
+      <c r="V13" s="129" t="n">
         <f aca="false">V11*2</f>
         <v>60</v>
       </c>
-      <c r="W13" s="128" t="n">
+      <c r="W13" s="129" t="n">
         <f aca="false">W11*2</f>
         <v>50</v>
       </c>
-      <c r="X13" s="128" t="n">
+      <c r="X13" s="129" t="n">
         <f aca="false">X11*2</f>
         <v>50</v>
       </c>
-      <c r="Y13" s="128" t="n">
+      <c r="Y13" s="129" t="n">
         <f aca="false">Y11*2</f>
         <v>20</v>
       </c>
-      <c r="Z13" s="128" t="n">
+      <c r="Z13" s="129" t="n">
         <f aca="false">Z11*2</f>
         <v>20</v>
       </c>
-      <c r="AA13" s="128" t="n">
+      <c r="AA13" s="129" t="n">
         <f aca="false">AA11*2</f>
         <v>60</v>
       </c>
-      <c r="AB13" s="128" t="n">
+      <c r="AB13" s="129" t="n">
         <f aca="false">AB11*2</f>
         <v>20</v>
       </c>
-      <c r="AC13" s="129" t="n">
+      <c r="AC13" s="130" t="n">
         <f aca="false">SUM(Q13:AB13)</f>
         <v>280</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="110" t="n">
+      <c r="A14" s="111" t="n">
         <v>59</v>
       </c>
-      <c r="B14" s="110" t="s">
+      <c r="B14" s="111" t="s">
         <v>8</v>
       </c>
       <c r="F14" s="5"/>
@@ -13505,7 +13522,7 @@
       <c r="I14" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="J14" s="120" t="n">
+      <c r="J14" s="121" t="n">
         <v>500</v>
       </c>
       <c r="K14" s="5" t="n">
@@ -13518,10 +13535,10 @@
       <c r="M14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="119" t="s">
+      <c r="A15" s="120" t="s">
         <v>186</v>
       </c>
-      <c r="B15" s="110" t="s">
+      <c r="B15" s="111" t="s">
         <v>7</v>
       </c>
       <c r="F15" s="5" t="n">
@@ -13553,7 +13570,7 @@
       <c r="M15" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="N15" s="118" t="s">
+      <c r="N15" s="119" t="s">
         <v>187</v>
       </c>
       <c r="O15" s="5" t="n">
@@ -13562,10 +13579,10 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="119" t="s">
+      <c r="A16" s="120" t="s">
         <v>186</v>
       </c>
-      <c r="B16" s="110" t="s">
+      <c r="B16" s="111" t="s">
         <v>7</v>
       </c>
       <c r="F16" s="5" t="n">
@@ -13598,7 +13615,7 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="110" t="s">
+      <c r="A17" s="111" t="s">
         <v>188</v>
       </c>
       <c r="F17" s="5"/>
@@ -13622,10 +13639,10 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="130" t="n">
+      <c r="A18" s="131" t="n">
         <v>305</v>
       </c>
-      <c r="B18" s="110" t="s">
+      <c r="B18" s="111" t="s">
         <v>8</v>
       </c>
       <c r="F18" s="5"/>
@@ -13647,15 +13664,15 @@
       <c r="M18" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="N18" s="111" t="s">
+      <c r="N18" s="112" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="130" t="n">
+      <c r="A19" s="131" t="n">
         <v>305</v>
       </c>
-      <c r="B19" s="110" t="s">
+      <c r="B19" s="111" t="s">
         <v>8</v>
       </c>
       <c r="F19" s="5"/>
@@ -13679,10 +13696,10 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="130" t="n">
+      <c r="A20" s="131" t="n">
         <v>305</v>
       </c>
-      <c r="B20" s="110" t="s">
+      <c r="B20" s="111" t="s">
         <v>8</v>
       </c>
       <c r="F20" s="5"/>
@@ -13706,17 +13723,17 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="131" t="s">
+      <c r="A21" s="132" t="s">
         <v>190</v>
       </c>
-      <c r="B21" s="110" t="n">
+      <c r="B21" s="111" t="n">
         <v>2025</v>
       </c>
-      <c r="C21" s="132"/>
+      <c r="C21" s="133"/>
       <c r="D21" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="E21" s="132"/>
+      <c r="E21" s="133"/>
       <c r="F21" s="5" t="n">
         <f aca="false">SUM(C21:E21)</f>
         <v>20</v>
@@ -13731,7 +13748,7 @@
       <c r="I21" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="J21" s="120" t="n">
+      <c r="J21" s="121" t="n">
         <v>100</v>
       </c>
       <c r="K21" s="5" t="n">
@@ -13745,22 +13762,22 @@
       <c r="M21" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="N21" s="118" t="s">
+      <c r="N21" s="119" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="131" t="s">
+      <c r="A22" s="132" t="s">
         <v>192</v>
       </c>
-      <c r="B22" s="110" t="n">
+      <c r="B22" s="111" t="n">
         <v>2025</v>
       </c>
-      <c r="C22" s="132"/>
+      <c r="C22" s="133"/>
       <c r="D22" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="E22" s="132"/>
+      <c r="E22" s="133"/>
       <c r="F22" s="5" t="n">
         <f aca="false">SUM(C22:E22)</f>
         <v>20</v>
@@ -13775,7 +13792,7 @@
       <c r="I22" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="J22" s="120" t="n">
+      <c r="J22" s="121" t="n">
         <v>100</v>
       </c>
       <c r="K22" s="5" t="n">
@@ -13789,15 +13806,15 @@
       <c r="M22" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="N22" s="118" t="s">
+      <c r="N22" s="119" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="110" t="s">
+      <c r="A23" s="111" t="s">
         <v>193</v>
       </c>
-      <c r="B23" s="110" t="s">
+      <c r="B23" s="111" t="s">
         <v>10</v>
       </c>
       <c r="F23" s="5"/>
@@ -13806,7 +13823,7 @@
       <c r="I23" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="J23" s="120" t="n">
+      <c r="J23" s="121" t="n">
         <v>200</v>
       </c>
       <c r="K23" s="5" t="n">
@@ -13821,10 +13838,10 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="110" t="s">
+      <c r="A24" s="111" t="s">
         <v>194</v>
       </c>
-      <c r="B24" s="110" t="s">
+      <c r="B24" s="111" t="s">
         <v>10</v>
       </c>
       <c r="F24" s="5"/>
@@ -13833,7 +13850,7 @@
       <c r="I24" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="J24" s="120" t="n">
+      <c r="J24" s="121" t="n">
         <v>50</v>
       </c>
       <c r="K24" s="5" t="n">
@@ -13848,10 +13865,10 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="110" t="s">
+      <c r="A25" s="111" t="s">
         <v>195</v>
       </c>
-      <c r="B25" s="110" t="s">
+      <c r="B25" s="111" t="s">
         <v>8</v>
       </c>
       <c r="F25" s="5"/>
@@ -13860,7 +13877,7 @@
       <c r="I25" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="J25" s="120" t="n">
+      <c r="J25" s="121" t="n">
         <f aca="false">10*6</f>
         <v>60</v>
       </c>
@@ -13876,17 +13893,17 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="110" t="s">
+      <c r="A26" s="111" t="s">
         <v>196</v>
       </c>
-      <c r="B26" s="110" t="s">
+      <c r="B26" s="111" t="s">
         <v>8</v>
       </c>
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
-      <c r="J26" s="120" t="n">
+      <c r="J26" s="121" t="n">
         <v>350</v>
       </c>
       <c r="K26" s="5" t="n">
@@ -13901,10 +13918,10 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="110" t="s">
+      <c r="A27" s="111" t="s">
         <v>197</v>
       </c>
-      <c r="B27" s="110" t="s">
+      <c r="B27" s="111" t="s">
         <v>8</v>
       </c>
       <c r="F27" s="5"/>
@@ -13920,7 +13937,7 @@
         <v>0</v>
       </c>
       <c r="M27" s="5"/>
-      <c r="N27" s="111" t="s">
+      <c r="N27" s="112" t="s">
         <v>199</v>
       </c>
       <c r="O27" s="5" t="s">
@@ -13928,10 +13945,10 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="110" t="s">
+      <c r="A28" s="111" t="s">
         <v>201</v>
       </c>
-      <c r="B28" s="110" t="s">
+      <c r="B28" s="111" t="s">
         <v>10</v>
       </c>
       <c r="F28" s="5"/>
@@ -13947,10 +13964,10 @@
       <c r="M28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="133" t="s">
+      <c r="A29" s="134" t="s">
         <v>202</v>
       </c>
-      <c r="B29" s="110" t="s">
+      <c r="B29" s="111" t="s">
         <v>9</v>
       </c>
       <c r="F29" s="5"/>
@@ -13966,10 +13983,10 @@
       <c r="M29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="110" t="s">
+      <c r="A30" s="111" t="s">
         <v>203</v>
       </c>
-      <c r="B30" s="110" t="s">
+      <c r="B30" s="111" t="s">
         <v>12</v>
       </c>
       <c r="F30" s="5"/>
@@ -13985,10 +14002,10 @@
       <c r="M30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="110" t="s">
+      <c r="A31" s="111" t="s">
         <v>204</v>
       </c>
-      <c r="B31" s="110" t="s">
+      <c r="B31" s="111" t="s">
         <v>9</v>
       </c>
       <c r="F31" s="5"/>
@@ -14004,10 +14021,10 @@
       <c r="M31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="110" t="s">
+      <c r="A32" s="111" t="s">
         <v>205</v>
       </c>
-      <c r="B32" s="110" t="s">
+      <c r="B32" s="111" t="s">
         <v>11</v>
       </c>
       <c r="F32" s="5"/>
@@ -14025,10 +14042,10 @@
       <c r="M32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="110" t="s">
+      <c r="A33" s="111" t="s">
         <v>206</v>
       </c>
-      <c r="B33" s="110" t="s">
+      <c r="B33" s="111" t="s">
         <v>6</v>
       </c>
       <c r="F33" s="5"/>
@@ -14044,7 +14061,7 @@
       <c r="M33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="110" t="s">
+      <c r="A34" s="111" t="s">
         <v>207</v>
       </c>
       <c r="F34" s="5"/>
@@ -14066,12 +14083,12 @@
       <c r="M34" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="N34" s="111" t="s">
+      <c r="N34" s="112" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="110" t="s">
+      <c r="A35" s="111" t="s">
         <v>209</v>
       </c>
       <c r="F35" s="5"/>
@@ -14093,7 +14110,7 @@
       <c r="M35" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="N35" s="111" t="s">
+      <c r="N35" s="112" t="s">
         <v>210</v>
       </c>
     </row>
@@ -14153,14 +14170,14 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
-      <c r="H41" s="117" t="n">
+      <c r="H41" s="118" t="n">
         <f aca="false">SUM(H3:H40)</f>
         <v>330000</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
       <c r="K41" s="5"/>
-      <c r="L41" s="117" t="n">
+      <c r="L41" s="118" t="n">
         <f aca="false">SUM(L3:L40)</f>
         <v>1434906</v>
       </c>
@@ -14187,7 +14204,7 @@
       <c r="M43" s="5"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="114" t="s">
+      <c r="A44" s="115" t="s">
         <v>198</v>
       </c>
       <c r="F44" s="5"/>
@@ -14200,10 +14217,10 @@
       <c r="M44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="110" t="n">
+      <c r="A45" s="111" t="n">
         <v>56</v>
       </c>
-      <c r="B45" s="110" t="s">
+      <c r="B45" s="111" t="s">
         <v>5</v>
       </c>
       <c r="F45" s="5"/>
@@ -14216,10 +14233,10 @@
       <c r="M45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="110" t="n">
+      <c r="A46" s="111" t="n">
         <v>202</v>
       </c>
-      <c r="B46" s="110" t="s">
+      <c r="B46" s="111" t="s">
         <v>5</v>
       </c>
       <c r="F46" s="5"/>
@@ -14232,10 +14249,10 @@
       <c r="M46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="110" t="n">
+      <c r="A47" s="111" t="n">
         <v>376</v>
       </c>
-      <c r="B47" s="110" t="s">
+      <c r="B47" s="111" t="s">
         <v>6</v>
       </c>
       <c r="F47" s="5"/>
@@ -14248,10 +14265,10 @@
       <c r="M47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="110" t="s">
+      <c r="A48" s="111" t="s">
         <v>211</v>
       </c>
-      <c r="B48" s="110" t="s">
+      <c r="B48" s="111" t="s">
         <v>15</v>
       </c>
       <c r="F48" s="5"/>
@@ -14264,10 +14281,10 @@
       <c r="M48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="110" t="s">
+      <c r="A49" s="111" t="s">
         <v>212</v>
       </c>
-      <c r="B49" s="110" t="s">
+      <c r="B49" s="111" t="s">
         <v>7</v>
       </c>
       <c r="F49" s="5"/>
@@ -14280,10 +14297,10 @@
       <c r="M49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="110" t="s">
+      <c r="A50" s="111" t="s">
         <v>213</v>
       </c>
-      <c r="B50" s="110" t="s">
+      <c r="B50" s="111" t="s">
         <v>6</v>
       </c>
       <c r="F50" s="5"/>
@@ -14317,48 +14334,48 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F53" s="5"/>
-      <c r="G53" s="117"/>
-      <c r="H53" s="117"/>
+      <c r="G53" s="118"/>
+      <c r="H53" s="118"/>
       <c r="I53" s="5"/>
       <c r="J53" s="5"/>
       <c r="K53" s="5"/>
-      <c r="L53" s="117"/>
+      <c r="L53" s="118"/>
       <c r="M53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="132"/>
+      <c r="A54" s="133"/>
       <c r="F54" s="5"/>
-      <c r="G54" s="117"/>
+      <c r="G54" s="118"/>
       <c r="H54" s="5"/>
       <c r="I54" s="5"/>
       <c r="J54" s="5"/>
       <c r="K54" s="5"/>
-      <c r="L54" s="117"/>
+      <c r="L54" s="118"/>
       <c r="M54" s="5"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="134"/>
+      <c r="A55" s="135"/>
       <c r="F55" s="5"/>
       <c r="G55" s="5"/>
       <c r="H55" s="5"/>
       <c r="I55" s="5"/>
       <c r="J55" s="5"/>
       <c r="K55" s="5"/>
-      <c r="L55" s="117"/>
+      <c r="L55" s="118"/>
       <c r="M55" s="5"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F56" s="5"/>
-      <c r="G56" s="135" t="n">
+      <c r="G56" s="136" t="n">
         <v>2025</v>
       </c>
-      <c r="H56" s="135" t="n">
+      <c r="H56" s="136" t="n">
         <v>2026</v>
       </c>
       <c r="I56" s="5"/>
       <c r="J56" s="5"/>
       <c r="K56" s="5"/>
-      <c r="L56" s="117"/>
+      <c r="L56" s="118"/>
       <c r="M56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14372,18 +14389,18 @@
       <c r="M57" s="5"/>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="110" t="s">
+      <c r="A58" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="C58" s="136" t="n">
+      <c r="C58" s="137" t="n">
         <f aca="false">$G$5*C5</f>
         <v>0</v>
       </c>
-      <c r="D58" s="136" t="n">
+      <c r="D58" s="137" t="n">
         <f aca="false">$G$5*D5</f>
         <v>30000</v>
       </c>
-      <c r="E58" s="136" t="n">
+      <c r="E58" s="137" t="n">
         <f aca="false">$G$5*E5</f>
         <v>0</v>
       </c>
@@ -14403,18 +14420,18 @@
       <c r="M58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="110" t="s">
+      <c r="A59" s="111" t="s">
         <v>38</v>
       </c>
-      <c r="C59" s="136" t="n">
+      <c r="C59" s="137" t="n">
         <f aca="false">$G$3*C3+$G$4*C4+$G$21*C21+$G$22*C22</f>
         <v>87000</v>
       </c>
-      <c r="D59" s="136" t="n">
+      <c r="D59" s="137" t="n">
         <f aca="false">$G$3*D3+$G$4*D4+$G$21*D21+$G$22*D22</f>
         <v>166000</v>
       </c>
-      <c r="E59" s="136" t="n">
+      <c r="E59" s="137" t="n">
         <f aca="false">$G$3*E3+$G$4*E4+$G$21*E21+$G$22*E22</f>
         <v>47000</v>
       </c>
@@ -14434,7 +14451,7 @@
       <c r="M59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="110" t="s">
+      <c r="A60" s="111" t="s">
         <v>35</v>
       </c>
       <c r="F60" s="5"/>
@@ -14461,11 +14478,11 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F62" s="5"/>
-      <c r="G62" s="117" t="n">
+      <c r="G62" s="118" t="n">
         <f aca="false">SUM(G58:G60)</f>
         <v>330000</v>
       </c>
-      <c r="H62" s="117" t="n">
+      <c r="H62" s="118" t="n">
         <f aca="false">SUM(H58:H60)</f>
         <v>1359906</v>
       </c>
@@ -14667,902 +14684,902 @@
   <dimension ref="A1:S35"/>
   <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="18" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="137" width="3.25"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="2" min="2" style="138" width="13.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="139" width="19.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="139" width="35.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="139" width="15.62"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="6" min="6" style="139" width="10.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="139" width="8.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="8" style="140" width="6.88"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="20" style="140" width="11.75"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="138" width="3.25"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="2" min="2" style="139" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="140" width="19.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="140" width="35.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="140" width="15.62"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="6" min="6" style="140" width="10.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="140" width="8.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="8" style="141" width="6.88"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="20" style="141" width="11.75"/>
   </cols>
   <sheetData>
-    <row r="1" s="143" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="141"/>
-      <c r="B1" s="142" t="s">
+    <row r="1" s="144" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="142"/>
+      <c r="B1" s="143" t="s">
         <v>214</v>
       </c>
-      <c r="C1" s="142" t="s">
+      <c r="C1" s="143" t="s">
         <v>215</v>
       </c>
-      <c r="D1" s="142" t="s">
+      <c r="D1" s="143" t="s">
         <v>216</v>
       </c>
-      <c r="E1" s="142" t="s">
+      <c r="E1" s="143" t="s">
         <v>217</v>
       </c>
-      <c r="F1" s="142" t="s">
+      <c r="F1" s="143" t="s">
         <v>218</v>
       </c>
-      <c r="G1" s="142"/>
-      <c r="H1" s="142" t="s">
+      <c r="G1" s="143"/>
+      <c r="H1" s="143" t="s">
         <v>219</v>
       </c>
-      <c r="I1" s="142" t="s">
+      <c r="I1" s="143" t="s">
         <v>220</v>
       </c>
-      <c r="J1" s="142" t="s">
+      <c r="J1" s="143" t="s">
         <v>221</v>
       </c>
-      <c r="K1" s="142" t="s">
+      <c r="K1" s="143" t="s">
         <v>222</v>
       </c>
-      <c r="L1" s="142" t="s">
+      <c r="L1" s="143" t="s">
         <v>223</v>
       </c>
-      <c r="M1" s="142" t="s">
+      <c r="M1" s="143" t="s">
         <v>224</v>
       </c>
-      <c r="N1" s="142" t="s">
+      <c r="N1" s="143" t="s">
         <v>225</v>
       </c>
-      <c r="O1" s="142" t="s">
+      <c r="O1" s="143" t="s">
         <v>226</v>
       </c>
-      <c r="P1" s="142" t="s">
+      <c r="P1" s="143" t="s">
         <v>227</v>
       </c>
-      <c r="Q1" s="142" t="s">
+      <c r="Q1" s="143" t="s">
         <v>228</v>
       </c>
-      <c r="R1" s="142" t="s">
+      <c r="R1" s="143" t="s">
         <v>229</v>
       </c>
-      <c r="S1" s="142" t="s">
+      <c r="S1" s="143" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C2" s="144" t="n">
+      <c r="C2" s="145" t="n">
         <v>56</v>
       </c>
-      <c r="D2" s="145" t="s">
+      <c r="D2" s="146" t="s">
         <v>231</v>
       </c>
-      <c r="E2" s="145" t="s">
+      <c r="E2" s="146" t="s">
         <v>232</v>
       </c>
-      <c r="F2" s="145" t="s">
+      <c r="F2" s="146" t="s">
         <v>233</v>
       </c>
-      <c r="G2" s="146" t="s">
+      <c r="G2" s="147" t="s">
         <v>234</v>
       </c>
-      <c r="H2" s="147"/>
-      <c r="I2" s="147" t="s">
+      <c r="H2" s="148"/>
+      <c r="I2" s="148" t="s">
         <v>235</v>
       </c>
-      <c r="J2" s="146"/>
-      <c r="K2" s="146"/>
-      <c r="L2" s="146"/>
-      <c r="M2" s="146"/>
-      <c r="N2" s="146"/>
-      <c r="O2" s="146"/>
-      <c r="P2" s="146"/>
-      <c r="Q2" s="146"/>
-      <c r="R2" s="146"/>
-      <c r="S2" s="146"/>
+      <c r="J2" s="147"/>
+      <c r="K2" s="147"/>
+      <c r="L2" s="147"/>
+      <c r="M2" s="147"/>
+      <c r="N2" s="147"/>
+      <c r="O2" s="147"/>
+      <c r="P2" s="147"/>
+      <c r="Q2" s="147"/>
+      <c r="R2" s="147"/>
+      <c r="S2" s="147"/>
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="148"/>
-      <c r="B3" s="149"/>
-      <c r="C3" s="144" t="n">
+      <c r="A3" s="149"/>
+      <c r="B3" s="150"/>
+      <c r="C3" s="145" t="n">
         <v>202</v>
       </c>
-      <c r="D3" s="145" t="s">
+      <c r="D3" s="146" t="s">
         <v>231</v>
       </c>
-      <c r="E3" s="145" t="s">
+      <c r="E3" s="146" t="s">
         <v>232</v>
       </c>
-      <c r="F3" s="145" t="s">
+      <c r="F3" s="146" t="s">
         <v>236</v>
       </c>
-      <c r="G3" s="146" t="s">
+      <c r="G3" s="147" t="s">
         <v>234</v>
       </c>
-      <c r="H3" s="147"/>
-      <c r="I3" s="147" t="s">
+      <c r="H3" s="148"/>
+      <c r="I3" s="148" t="s">
         <v>235</v>
       </c>
-      <c r="J3" s="146"/>
-      <c r="K3" s="146"/>
-      <c r="L3" s="146"/>
-      <c r="M3" s="146"/>
-      <c r="N3" s="146"/>
-      <c r="O3" s="146"/>
-      <c r="P3" s="146"/>
-      <c r="Q3" s="146"/>
-      <c r="R3" s="146"/>
-      <c r="S3" s="146"/>
+      <c r="J3" s="147"/>
+      <c r="K3" s="147"/>
+      <c r="L3" s="147"/>
+      <c r="M3" s="147"/>
+      <c r="N3" s="147"/>
+      <c r="O3" s="147"/>
+      <c r="P3" s="147"/>
+      <c r="Q3" s="147"/>
+      <c r="R3" s="147"/>
+      <c r="S3" s="147"/>
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="148" t="n">
+      <c r="A4" s="149" t="n">
         <v>12</v>
       </c>
-      <c r="B4" s="149"/>
-      <c r="C4" s="144" t="n">
+      <c r="B4" s="150"/>
+      <c r="C4" s="145" t="n">
         <v>376</v>
       </c>
-      <c r="D4" s="145" t="s">
+      <c r="D4" s="146" t="s">
         <v>237</v>
       </c>
-      <c r="E4" s="145" t="s">
+      <c r="E4" s="146" t="s">
         <v>198</v>
       </c>
-      <c r="F4" s="145"/>
-      <c r="G4" s="145"/>
-      <c r="H4" s="147"/>
-      <c r="I4" s="147"/>
-      <c r="J4" s="147"/>
-      <c r="K4" s="146"/>
-      <c r="L4" s="146"/>
-      <c r="M4" s="146"/>
-      <c r="N4" s="146"/>
-      <c r="O4" s="146"/>
-      <c r="P4" s="146"/>
-      <c r="Q4" s="146"/>
-      <c r="R4" s="146"/>
-      <c r="S4" s="146"/>
+      <c r="F4" s="146"/>
+      <c r="G4" s="146"/>
+      <c r="H4" s="148"/>
+      <c r="I4" s="148"/>
+      <c r="J4" s="148"/>
+      <c r="K4" s="147"/>
+      <c r="L4" s="147"/>
+      <c r="M4" s="147"/>
+      <c r="N4" s="147"/>
+      <c r="O4" s="147"/>
+      <c r="P4" s="147"/>
+      <c r="Q4" s="147"/>
+      <c r="R4" s="147"/>
+      <c r="S4" s="147"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="148" t="n">
+      <c r="A5" s="149" t="n">
         <v>13</v>
       </c>
-      <c r="B5" s="149"/>
-      <c r="C5" s="144" t="n">
+      <c r="B5" s="150"/>
+      <c r="C5" s="145" t="n">
         <v>305</v>
       </c>
-      <c r="D5" s="145" t="s">
+      <c r="D5" s="146" t="s">
         <v>238</v>
       </c>
-      <c r="E5" s="145" t="s">
+      <c r="E5" s="146" t="s">
         <v>232</v>
       </c>
-      <c r="F5" s="145"/>
-      <c r="G5" s="145"/>
-      <c r="H5" s="147"/>
-      <c r="I5" s="147"/>
-      <c r="J5" s="147"/>
-      <c r="K5" s="147"/>
-      <c r="L5" s="147"/>
-      <c r="M5" s="146"/>
-      <c r="N5" s="146"/>
-      <c r="O5" s="146"/>
-      <c r="P5" s="146"/>
-      <c r="Q5" s="146"/>
-      <c r="R5" s="146"/>
-      <c r="S5" s="146"/>
+      <c r="F5" s="146"/>
+      <c r="G5" s="146"/>
+      <c r="H5" s="148"/>
+      <c r="I5" s="148"/>
+      <c r="J5" s="148"/>
+      <c r="K5" s="148"/>
+      <c r="L5" s="148"/>
+      <c r="M5" s="147"/>
+      <c r="N5" s="147"/>
+      <c r="O5" s="147"/>
+      <c r="P5" s="147"/>
+      <c r="Q5" s="147"/>
+      <c r="R5" s="147"/>
+      <c r="S5" s="147"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="148"/>
-      <c r="B6" s="149"/>
-      <c r="C6" s="144" t="s">
+      <c r="A6" s="149"/>
+      <c r="B6" s="150"/>
+      <c r="C6" s="145" t="s">
         <v>239</v>
       </c>
-      <c r="D6" s="145" t="s">
+      <c r="D6" s="146" t="s">
         <v>240</v>
       </c>
-      <c r="E6" s="145"/>
-      <c r="F6" s="145"/>
-      <c r="G6" s="145"/>
-      <c r="H6" s="147"/>
-      <c r="I6" s="147"/>
-      <c r="J6" s="147"/>
-      <c r="K6" s="147"/>
-      <c r="L6" s="147"/>
-      <c r="M6" s="146"/>
-      <c r="N6" s="146"/>
-      <c r="O6" s="146"/>
-      <c r="P6" s="146"/>
-      <c r="Q6" s="146"/>
-      <c r="R6" s="146"/>
-      <c r="S6" s="146"/>
+      <c r="E6" s="146"/>
+      <c r="F6" s="146"/>
+      <c r="G6" s="146"/>
+      <c r="H6" s="148"/>
+      <c r="I6" s="148"/>
+      <c r="J6" s="148"/>
+      <c r="K6" s="148"/>
+      <c r="L6" s="148"/>
+      <c r="M6" s="147"/>
+      <c r="N6" s="147"/>
+      <c r="O6" s="147"/>
+      <c r="P6" s="147"/>
+      <c r="Q6" s="147"/>
+      <c r="R6" s="147"/>
+      <c r="S6" s="147"/>
     </row>
     <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="148" t="n">
+      <c r="A7" s="149" t="n">
         <v>17</v>
       </c>
-      <c r="B7" s="150"/>
-      <c r="C7" s="151" t="s">
+      <c r="B7" s="151"/>
+      <c r="C7" s="152" t="s">
         <v>241</v>
       </c>
-      <c r="D7" s="152" t="s">
+      <c r="D7" s="153" t="s">
         <v>242</v>
       </c>
-      <c r="E7" s="152" t="s">
+      <c r="E7" s="153" t="s">
         <v>158</v>
       </c>
-      <c r="F7" s="152"/>
-      <c r="G7" s="152"/>
-      <c r="H7" s="147"/>
-      <c r="I7" s="147"/>
-      <c r="J7" s="147"/>
-      <c r="K7" s="147"/>
-      <c r="L7" s="147"/>
-      <c r="M7" s="146"/>
-      <c r="N7" s="146"/>
-      <c r="O7" s="146"/>
-      <c r="P7" s="146"/>
-      <c r="Q7" s="146"/>
-      <c r="R7" s="146"/>
-      <c r="S7" s="146"/>
+      <c r="F7" s="153"/>
+      <c r="G7" s="153"/>
+      <c r="H7" s="148"/>
+      <c r="I7" s="148"/>
+      <c r="J7" s="148"/>
+      <c r="K7" s="148"/>
+      <c r="L7" s="148"/>
+      <c r="M7" s="147"/>
+      <c r="N7" s="147"/>
+      <c r="O7" s="147"/>
+      <c r="P7" s="147"/>
+      <c r="Q7" s="147"/>
+      <c r="R7" s="147"/>
+      <c r="S7" s="147"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="148" t="n">
+      <c r="A8" s="149" t="n">
         <v>18</v>
       </c>
-      <c r="B8" s="150"/>
-      <c r="C8" s="151" t="s">
+      <c r="B8" s="151"/>
+      <c r="C8" s="152" t="s">
         <v>243</v>
       </c>
-      <c r="D8" s="153" t="s">
+      <c r="D8" s="154" t="s">
         <v>244</v>
       </c>
-      <c r="E8" s="152" t="s">
+      <c r="E8" s="153" t="s">
         <v>158</v>
       </c>
-      <c r="F8" s="153"/>
-      <c r="G8" s="153"/>
-      <c r="H8" s="147"/>
-      <c r="I8" s="147"/>
-      <c r="J8" s="147"/>
-      <c r="K8" s="147"/>
-      <c r="L8" s="147"/>
-      <c r="M8" s="146"/>
-      <c r="N8" s="146"/>
-      <c r="O8" s="146"/>
-      <c r="P8" s="146"/>
-      <c r="Q8" s="146"/>
-      <c r="R8" s="146"/>
-      <c r="S8" s="146"/>
+      <c r="F8" s="154"/>
+      <c r="G8" s="154"/>
+      <c r="H8" s="148"/>
+      <c r="I8" s="148"/>
+      <c r="J8" s="148"/>
+      <c r="K8" s="148"/>
+      <c r="L8" s="148"/>
+      <c r="M8" s="147"/>
+      <c r="N8" s="147"/>
+      <c r="O8" s="147"/>
+      <c r="P8" s="147"/>
+      <c r="Q8" s="147"/>
+      <c r="R8" s="147"/>
+      <c r="S8" s="147"/>
     </row>
     <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="148" t="n">
+      <c r="A9" s="149" t="n">
         <v>20</v>
       </c>
-      <c r="B9" s="154"/>
-      <c r="C9" s="151" t="s">
+      <c r="B9" s="155"/>
+      <c r="C9" s="152" t="s">
         <v>245</v>
       </c>
-      <c r="D9" s="153" t="s">
+      <c r="D9" s="154" t="s">
         <v>244</v>
       </c>
-      <c r="E9" s="152" t="s">
+      <c r="E9" s="153" t="s">
         <v>158</v>
       </c>
-      <c r="F9" s="153"/>
-      <c r="G9" s="153"/>
-      <c r="H9" s="147"/>
-      <c r="I9" s="147"/>
-      <c r="J9" s="147"/>
-      <c r="K9" s="147"/>
-      <c r="L9" s="147"/>
-      <c r="M9" s="146"/>
-      <c r="N9" s="146"/>
-      <c r="O9" s="146"/>
-      <c r="P9" s="146"/>
-      <c r="Q9" s="146"/>
-      <c r="R9" s="146"/>
-      <c r="S9" s="146"/>
+      <c r="F9" s="154"/>
+      <c r="G9" s="154"/>
+      <c r="H9" s="148"/>
+      <c r="I9" s="148"/>
+      <c r="J9" s="148"/>
+      <c r="K9" s="148"/>
+      <c r="L9" s="148"/>
+      <c r="M9" s="147"/>
+      <c r="N9" s="147"/>
+      <c r="O9" s="147"/>
+      <c r="P9" s="147"/>
+      <c r="Q9" s="147"/>
+      <c r="R9" s="147"/>
+      <c r="S9" s="147"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="155" t="n">
+      <c r="A10" s="156" t="n">
         <v>27</v>
       </c>
-      <c r="B10" s="149"/>
-      <c r="C10" s="151" t="s">
+      <c r="B10" s="150"/>
+      <c r="C10" s="152" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="153" t="s">
+      <c r="D10" s="154" t="s">
         <v>246</v>
       </c>
-      <c r="E10" s="152" t="s">
+      <c r="E10" s="153" t="s">
         <v>158</v>
       </c>
-      <c r="F10" s="153"/>
-      <c r="G10" s="153"/>
-      <c r="H10" s="147"/>
-      <c r="I10" s="147"/>
-      <c r="J10" s="147"/>
-      <c r="K10" s="147"/>
-      <c r="L10" s="147"/>
-      <c r="M10" s="147"/>
-      <c r="N10" s="147"/>
-      <c r="O10" s="146"/>
-      <c r="P10" s="146"/>
-      <c r="Q10" s="146"/>
-      <c r="R10" s="146"/>
-      <c r="S10" s="146"/>
+      <c r="F10" s="154"/>
+      <c r="G10" s="154"/>
+      <c r="H10" s="148"/>
+      <c r="I10" s="148"/>
+      <c r="J10" s="148"/>
+      <c r="K10" s="148"/>
+      <c r="L10" s="148"/>
+      <c r="M10" s="148"/>
+      <c r="N10" s="148"/>
+      <c r="O10" s="147"/>
+      <c r="P10" s="147"/>
+      <c r="Q10" s="147"/>
+      <c r="R10" s="147"/>
+      <c r="S10" s="147"/>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="137" t="n">
+      <c r="A11" s="138" t="n">
         <v>28</v>
       </c>
-      <c r="B11" s="149"/>
-      <c r="C11" s="151" t="s">
+      <c r="B11" s="150"/>
+      <c r="C11" s="152" t="s">
         <v>194</v>
       </c>
-      <c r="D11" s="153" t="s">
+      <c r="D11" s="154" t="s">
         <v>246</v>
       </c>
-      <c r="E11" s="152" t="s">
+      <c r="E11" s="153" t="s">
         <v>158</v>
       </c>
-      <c r="F11" s="153"/>
-      <c r="G11" s="153"/>
-      <c r="H11" s="147"/>
-      <c r="I11" s="147"/>
-      <c r="J11" s="147"/>
-      <c r="K11" s="147"/>
-      <c r="L11" s="147"/>
-      <c r="M11" s="147"/>
-      <c r="N11" s="147"/>
-      <c r="O11" s="146"/>
-      <c r="P11" s="146"/>
-      <c r="Q11" s="146"/>
-      <c r="R11" s="146"/>
-      <c r="S11" s="146"/>
+      <c r="F11" s="154"/>
+      <c r="G11" s="154"/>
+      <c r="H11" s="148"/>
+      <c r="I11" s="148"/>
+      <c r="J11" s="148"/>
+      <c r="K11" s="148"/>
+      <c r="L11" s="148"/>
+      <c r="M11" s="148"/>
+      <c r="N11" s="148"/>
+      <c r="O11" s="147"/>
+      <c r="P11" s="147"/>
+      <c r="Q11" s="147"/>
+      <c r="R11" s="147"/>
+      <c r="S11" s="147"/>
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="137" t="n">
+      <c r="A12" s="138" t="n">
         <v>29</v>
       </c>
-      <c r="B12" s="149"/>
-      <c r="C12" s="151" t="s">
+      <c r="B12" s="150"/>
+      <c r="C12" s="152" t="s">
         <v>195</v>
       </c>
-      <c r="D12" s="153" t="s">
+      <c r="D12" s="154" t="s">
         <v>247</v>
       </c>
-      <c r="E12" s="152" t="s">
+      <c r="E12" s="153" t="s">
         <v>158</v>
       </c>
-      <c r="F12" s="153"/>
-      <c r="G12" s="153"/>
-      <c r="H12" s="147"/>
-      <c r="I12" s="147"/>
-      <c r="J12" s="147"/>
-      <c r="K12" s="147"/>
-      <c r="L12" s="147"/>
-      <c r="M12" s="146"/>
-      <c r="N12" s="146"/>
-      <c r="O12" s="146"/>
-      <c r="P12" s="146"/>
-      <c r="Q12" s="146"/>
-      <c r="R12" s="146"/>
-      <c r="S12" s="146"/>
+      <c r="F12" s="154"/>
+      <c r="G12" s="154"/>
+      <c r="H12" s="148"/>
+      <c r="I12" s="148"/>
+      <c r="J12" s="148"/>
+      <c r="K12" s="148"/>
+      <c r="L12" s="148"/>
+      <c r="M12" s="147"/>
+      <c r="N12" s="147"/>
+      <c r="O12" s="147"/>
+      <c r="P12" s="147"/>
+      <c r="Q12" s="147"/>
+      <c r="R12" s="147"/>
+      <c r="S12" s="147"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="149"/>
-      <c r="C13" s="151" t="s">
+      <c r="B13" s="150"/>
+      <c r="C13" s="152" t="s">
         <v>196</v>
       </c>
-      <c r="D13" s="153" t="s">
+      <c r="D13" s="154" t="s">
         <v>248</v>
       </c>
-      <c r="E13" s="152" t="s">
+      <c r="E13" s="153" t="s">
         <v>158</v>
       </c>
-      <c r="F13" s="153"/>
-      <c r="G13" s="153"/>
-      <c r="H13" s="147"/>
-      <c r="I13" s="147"/>
-      <c r="J13" s="147"/>
-      <c r="K13" s="147"/>
-      <c r="L13" s="147"/>
-      <c r="M13" s="146"/>
-      <c r="N13" s="146"/>
-      <c r="O13" s="146"/>
-      <c r="P13" s="146"/>
-      <c r="Q13" s="146"/>
-      <c r="R13" s="146"/>
-      <c r="S13" s="146"/>
+      <c r="F13" s="154"/>
+      <c r="G13" s="154"/>
+      <c r="H13" s="148"/>
+      <c r="I13" s="148"/>
+      <c r="J13" s="148"/>
+      <c r="K13" s="148"/>
+      <c r="L13" s="148"/>
+      <c r="M13" s="147"/>
+      <c r="N13" s="147"/>
+      <c r="O13" s="147"/>
+      <c r="P13" s="147"/>
+      <c r="Q13" s="147"/>
+      <c r="R13" s="147"/>
+      <c r="S13" s="147"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="149"/>
-      <c r="C14" s="144" t="s">
+      <c r="B14" s="150"/>
+      <c r="C14" s="145" t="s">
         <v>197</v>
       </c>
-      <c r="D14" s="153" t="s">
+      <c r="D14" s="154" t="s">
         <v>249</v>
       </c>
-      <c r="E14" s="152" t="s">
+      <c r="E14" s="153" t="s">
         <v>158</v>
       </c>
-      <c r="F14" s="153"/>
-      <c r="G14" s="153"/>
-      <c r="H14" s="147"/>
-      <c r="I14" s="147"/>
-      <c r="J14" s="147"/>
-      <c r="K14" s="147"/>
-      <c r="L14" s="147"/>
-      <c r="M14" s="146"/>
-      <c r="N14" s="146"/>
-      <c r="O14" s="146"/>
-      <c r="P14" s="146"/>
-      <c r="Q14" s="146"/>
-      <c r="R14" s="146"/>
-      <c r="S14" s="146"/>
+      <c r="F14" s="154"/>
+      <c r="G14" s="154"/>
+      <c r="H14" s="148"/>
+      <c r="I14" s="148"/>
+      <c r="J14" s="148"/>
+      <c r="K14" s="148"/>
+      <c r="L14" s="148"/>
+      <c r="M14" s="147"/>
+      <c r="N14" s="147"/>
+      <c r="O14" s="147"/>
+      <c r="P14" s="147"/>
+      <c r="Q14" s="147"/>
+      <c r="R14" s="147"/>
+      <c r="S14" s="147"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="149"/>
-      <c r="C15" s="144" t="s">
+      <c r="B15" s="150"/>
+      <c r="C15" s="145" t="s">
         <v>201</v>
       </c>
-      <c r="D15" s="153" t="s">
+      <c r="D15" s="154" t="s">
         <v>250</v>
       </c>
-      <c r="E15" s="152" t="s">
+      <c r="E15" s="153" t="s">
         <v>158</v>
       </c>
-      <c r="F15" s="153"/>
-      <c r="G15" s="153"/>
-      <c r="H15" s="147"/>
-      <c r="I15" s="147"/>
-      <c r="J15" s="147"/>
-      <c r="K15" s="147"/>
-      <c r="L15" s="147"/>
-      <c r="M15" s="147"/>
-      <c r="N15" s="147"/>
-      <c r="O15" s="146"/>
-      <c r="P15" s="146"/>
-      <c r="Q15" s="146"/>
-      <c r="R15" s="146"/>
-      <c r="S15" s="146"/>
+      <c r="F15" s="154"/>
+      <c r="G15" s="154"/>
+      <c r="H15" s="148"/>
+      <c r="I15" s="148"/>
+      <c r="J15" s="148"/>
+      <c r="K15" s="148"/>
+      <c r="L15" s="148"/>
+      <c r="M15" s="148"/>
+      <c r="N15" s="148"/>
+      <c r="O15" s="147"/>
+      <c r="P15" s="147"/>
+      <c r="Q15" s="147"/>
+      <c r="R15" s="147"/>
+      <c r="S15" s="147"/>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="149"/>
-      <c r="C16" s="156" t="s">
+      <c r="B16" s="150"/>
+      <c r="C16" s="157" t="s">
         <v>202</v>
       </c>
-      <c r="D16" s="157" t="s">
+      <c r="D16" s="158" t="s">
         <v>251</v>
       </c>
-      <c r="E16" s="157" t="s">
+      <c r="E16" s="158" t="s">
         <v>158</v>
       </c>
-      <c r="F16" s="157"/>
-      <c r="G16" s="157"/>
-      <c r="H16" s="147"/>
-      <c r="I16" s="147"/>
-      <c r="J16" s="147"/>
-      <c r="K16" s="147"/>
-      <c r="L16" s="147"/>
-      <c r="M16" s="147"/>
-      <c r="N16" s="146"/>
-      <c r="O16" s="146"/>
-      <c r="P16" s="146"/>
-      <c r="Q16" s="146"/>
-      <c r="R16" s="146"/>
-      <c r="S16" s="146"/>
+      <c r="F16" s="158"/>
+      <c r="G16" s="158"/>
+      <c r="H16" s="148"/>
+      <c r="I16" s="148"/>
+      <c r="J16" s="148"/>
+      <c r="K16" s="148"/>
+      <c r="L16" s="148"/>
+      <c r="M16" s="148"/>
+      <c r="N16" s="147"/>
+      <c r="O16" s="147"/>
+      <c r="P16" s="147"/>
+      <c r="Q16" s="147"/>
+      <c r="R16" s="147"/>
+      <c r="S16" s="147"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="148"/>
-      <c r="B17" s="149"/>
-      <c r="C17" s="151" t="s">
+      <c r="A17" s="149"/>
+      <c r="B17" s="150"/>
+      <c r="C17" s="152" t="s">
         <v>203</v>
       </c>
-      <c r="D17" s="145" t="s">
+      <c r="D17" s="146" t="s">
         <v>252</v>
       </c>
-      <c r="E17" s="145" t="s">
+      <c r="E17" s="146" t="s">
         <v>158</v>
       </c>
-      <c r="F17" s="145"/>
-      <c r="G17" s="145"/>
-      <c r="H17" s="146"/>
-      <c r="I17" s="146"/>
-      <c r="J17" s="147"/>
-      <c r="K17" s="147"/>
-      <c r="L17" s="147"/>
-      <c r="M17" s="147"/>
-      <c r="N17" s="147"/>
-      <c r="O17" s="147"/>
-      <c r="P17" s="147"/>
-      <c r="Q17" s="146"/>
-      <c r="R17" s="146"/>
-      <c r="S17" s="146"/>
+      <c r="F17" s="146"/>
+      <c r="G17" s="146"/>
+      <c r="H17" s="147"/>
+      <c r="I17" s="147"/>
+      <c r="J17" s="148"/>
+      <c r="K17" s="148"/>
+      <c r="L17" s="148"/>
+      <c r="M17" s="148"/>
+      <c r="N17" s="148"/>
+      <c r="O17" s="148"/>
+      <c r="P17" s="148"/>
+      <c r="Q17" s="147"/>
+      <c r="R17" s="147"/>
+      <c r="S17" s="147"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="149"/>
-      <c r="C18" s="158" t="s">
+      <c r="B18" s="150"/>
+      <c r="C18" s="159" t="s">
         <v>204</v>
       </c>
-      <c r="D18" s="153" t="s">
+      <c r="D18" s="154" t="s">
         <v>253</v>
       </c>
-      <c r="E18" s="153" t="s">
+      <c r="E18" s="154" t="s">
         <v>254</v>
       </c>
-      <c r="F18" s="153"/>
-      <c r="G18" s="153"/>
-      <c r="H18" s="147"/>
-      <c r="I18" s="147"/>
-      <c r="J18" s="147"/>
-      <c r="K18" s="147"/>
-      <c r="L18" s="147"/>
-      <c r="M18" s="147"/>
-      <c r="N18" s="146"/>
-      <c r="O18" s="146"/>
-      <c r="P18" s="146"/>
-      <c r="Q18" s="146"/>
-      <c r="R18" s="146"/>
-      <c r="S18" s="146"/>
+      <c r="F18" s="154"/>
+      <c r="G18" s="154"/>
+      <c r="H18" s="148"/>
+      <c r="I18" s="148"/>
+      <c r="J18" s="148"/>
+      <c r="K18" s="148"/>
+      <c r="L18" s="148"/>
+      <c r="M18" s="148"/>
+      <c r="N18" s="147"/>
+      <c r="O18" s="147"/>
+      <c r="P18" s="147"/>
+      <c r="Q18" s="147"/>
+      <c r="R18" s="147"/>
+      <c r="S18" s="147"/>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="149"/>
-      <c r="C19" s="144" t="s">
+      <c r="B19" s="150"/>
+      <c r="C19" s="145" t="s">
         <v>205</v>
       </c>
-      <c r="D19" s="153" t="s">
+      <c r="D19" s="154" t="s">
         <v>255</v>
       </c>
-      <c r="E19" s="153"/>
-      <c r="F19" s="153"/>
-      <c r="G19" s="153"/>
-      <c r="H19" s="146"/>
-      <c r="I19" s="146"/>
-      <c r="J19" s="147"/>
-      <c r="K19" s="147"/>
-      <c r="L19" s="147"/>
-      <c r="M19" s="147"/>
-      <c r="N19" s="147"/>
-      <c r="O19" s="147"/>
-      <c r="P19" s="146"/>
-      <c r="Q19" s="146"/>
-      <c r="R19" s="146"/>
-      <c r="S19" s="146"/>
+      <c r="E19" s="154"/>
+      <c r="F19" s="154"/>
+      <c r="G19" s="154"/>
+      <c r="H19" s="147"/>
+      <c r="I19" s="147"/>
+      <c r="J19" s="148"/>
+      <c r="K19" s="148"/>
+      <c r="L19" s="148"/>
+      <c r="M19" s="148"/>
+      <c r="N19" s="148"/>
+      <c r="O19" s="148"/>
+      <c r="P19" s="147"/>
+      <c r="Q19" s="147"/>
+      <c r="R19" s="147"/>
+      <c r="S19" s="147"/>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="149"/>
-      <c r="C20" s="144" t="s">
+      <c r="B20" s="150"/>
+      <c r="C20" s="145" t="s">
         <v>206</v>
       </c>
-      <c r="D20" s="153" t="s">
+      <c r="D20" s="154" t="s">
         <v>256</v>
       </c>
-      <c r="E20" s="153"/>
-      <c r="F20" s="153"/>
-      <c r="G20" s="153"/>
-      <c r="H20" s="147"/>
-      <c r="I20" s="147"/>
-      <c r="J20" s="147"/>
-      <c r="K20" s="146"/>
-      <c r="L20" s="146"/>
-      <c r="M20" s="146"/>
-      <c r="N20" s="146"/>
-      <c r="O20" s="146"/>
-      <c r="P20" s="146"/>
-      <c r="Q20" s="146"/>
-      <c r="R20" s="146"/>
-      <c r="S20" s="146"/>
+      <c r="E20" s="154"/>
+      <c r="F20" s="154"/>
+      <c r="G20" s="154"/>
+      <c r="H20" s="148"/>
+      <c r="I20" s="148"/>
+      <c r="J20" s="148"/>
+      <c r="K20" s="147"/>
+      <c r="L20" s="147"/>
+      <c r="M20" s="147"/>
+      <c r="N20" s="147"/>
+      <c r="O20" s="147"/>
+      <c r="P20" s="147"/>
+      <c r="Q20" s="147"/>
+      <c r="R20" s="147"/>
+      <c r="S20" s="147"/>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="149"/>
-      <c r="C21" s="144" t="s">
+      <c r="B21" s="150"/>
+      <c r="C21" s="145" t="s">
         <v>257</v>
       </c>
-      <c r="D21" s="153" t="s">
+      <c r="D21" s="154" t="s">
         <v>258</v>
       </c>
-      <c r="E21" s="153"/>
-      <c r="F21" s="153"/>
-      <c r="G21" s="153"/>
-      <c r="H21" s="147"/>
-      <c r="I21" s="147"/>
-      <c r="J21" s="147"/>
-      <c r="K21" s="146"/>
-      <c r="L21" s="146"/>
-      <c r="M21" s="146"/>
-      <c r="N21" s="146"/>
-      <c r="O21" s="146"/>
-      <c r="P21" s="146"/>
-      <c r="Q21" s="146"/>
-      <c r="R21" s="146"/>
-      <c r="S21" s="146"/>
+      <c r="E21" s="154"/>
+      <c r="F21" s="154"/>
+      <c r="G21" s="154"/>
+      <c r="H21" s="148"/>
+      <c r="I21" s="148"/>
+      <c r="J21" s="148"/>
+      <c r="K21" s="147"/>
+      <c r="L21" s="147"/>
+      <c r="M21" s="147"/>
+      <c r="N21" s="147"/>
+      <c r="O21" s="147"/>
+      <c r="P21" s="147"/>
+      <c r="Q21" s="147"/>
+      <c r="R21" s="147"/>
+      <c r="S21" s="147"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="149"/>
-      <c r="C22" s="144" t="s">
+      <c r="B22" s="150"/>
+      <c r="C22" s="145" t="s">
         <v>211</v>
       </c>
-      <c r="D22" s="153" t="s">
+      <c r="D22" s="154" t="s">
         <v>259</v>
       </c>
-      <c r="E22" s="153" t="s">
+      <c r="E22" s="154" t="s">
         <v>198</v>
       </c>
-      <c r="F22" s="153"/>
-      <c r="G22" s="153"/>
-      <c r="H22" s="147"/>
-      <c r="I22" s="147"/>
-      <c r="J22" s="147"/>
-      <c r="K22" s="147"/>
-      <c r="L22" s="147"/>
-      <c r="M22" s="147"/>
-      <c r="N22" s="147"/>
-      <c r="O22" s="147"/>
-      <c r="P22" s="147"/>
-      <c r="Q22" s="147"/>
-      <c r="R22" s="147"/>
-      <c r="S22" s="147"/>
+      <c r="F22" s="154"/>
+      <c r="G22" s="154"/>
+      <c r="H22" s="148"/>
+      <c r="I22" s="148"/>
+      <c r="J22" s="148"/>
+      <c r="K22" s="148"/>
+      <c r="L22" s="148"/>
+      <c r="M22" s="148"/>
+      <c r="N22" s="148"/>
+      <c r="O22" s="148"/>
+      <c r="P22" s="148"/>
+      <c r="Q22" s="148"/>
+      <c r="R22" s="148"/>
+      <c r="S22" s="148"/>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="149"/>
-      <c r="C23" s="144" t="s">
+      <c r="B23" s="150"/>
+      <c r="C23" s="145" t="s">
         <v>212</v>
       </c>
-      <c r="D23" s="153" t="s">
+      <c r="D23" s="154" t="s">
         <v>260</v>
       </c>
-      <c r="E23" s="153" t="s">
+      <c r="E23" s="154" t="s">
         <v>198</v>
       </c>
-      <c r="F23" s="153"/>
-      <c r="G23" s="153"/>
-      <c r="H23" s="147"/>
-      <c r="I23" s="147"/>
-      <c r="J23" s="147"/>
-      <c r="K23" s="147"/>
-      <c r="L23" s="146"/>
-      <c r="M23" s="146"/>
-      <c r="N23" s="146"/>
-      <c r="O23" s="146"/>
-      <c r="P23" s="146"/>
-      <c r="Q23" s="146"/>
-      <c r="R23" s="146"/>
-      <c r="S23" s="146"/>
+      <c r="F23" s="154"/>
+      <c r="G23" s="154"/>
+      <c r="H23" s="148"/>
+      <c r="I23" s="148"/>
+      <c r="J23" s="148"/>
+      <c r="K23" s="148"/>
+      <c r="L23" s="147"/>
+      <c r="M23" s="147"/>
+      <c r="N23" s="147"/>
+      <c r="O23" s="147"/>
+      <c r="P23" s="147"/>
+      <c r="Q23" s="147"/>
+      <c r="R23" s="147"/>
+      <c r="S23" s="147"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="149"/>
-      <c r="C24" s="144" t="s">
+      <c r="B24" s="150"/>
+      <c r="C24" s="145" t="s">
         <v>213</v>
       </c>
-      <c r="D24" s="153" t="s">
+      <c r="D24" s="154" t="s">
         <v>261</v>
       </c>
-      <c r="E24" s="153" t="s">
+      <c r="E24" s="154" t="s">
         <v>198</v>
       </c>
-      <c r="F24" s="153"/>
-      <c r="G24" s="153"/>
-      <c r="H24" s="147"/>
-      <c r="I24" s="147"/>
-      <c r="J24" s="147"/>
-      <c r="K24" s="146"/>
-      <c r="L24" s="146"/>
-      <c r="M24" s="146"/>
-      <c r="N24" s="146"/>
-      <c r="O24" s="146"/>
-      <c r="P24" s="146"/>
-      <c r="Q24" s="146"/>
-      <c r="R24" s="146"/>
-      <c r="S24" s="146"/>
+      <c r="F24" s="154"/>
+      <c r="G24" s="154"/>
+      <c r="H24" s="148"/>
+      <c r="I24" s="148"/>
+      <c r="J24" s="148"/>
+      <c r="K24" s="147"/>
+      <c r="L24" s="147"/>
+      <c r="M24" s="147"/>
+      <c r="N24" s="147"/>
+      <c r="O24" s="147"/>
+      <c r="P24" s="147"/>
+      <c r="Q24" s="147"/>
+      <c r="R24" s="147"/>
+      <c r="S24" s="147"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="149"/>
-      <c r="C25" s="144" t="s">
+      <c r="B25" s="150"/>
+      <c r="C25" s="145" t="s">
         <v>262</v>
       </c>
-      <c r="D25" s="153" t="s">
+      <c r="D25" s="154" t="s">
         <v>263</v>
       </c>
-      <c r="E25" s="139" t="s">
+      <c r="E25" s="140" t="s">
         <v>264</v>
       </c>
-      <c r="J25" s="147"/>
-      <c r="K25" s="147"/>
-      <c r="L25" s="147"/>
-      <c r="M25" s="147"/>
-      <c r="N25" s="147"/>
-      <c r="O25" s="147"/>
-      <c r="P25" s="147"/>
-      <c r="Q25" s="146"/>
-      <c r="R25" s="146"/>
-      <c r="S25" s="146"/>
+      <c r="J25" s="148"/>
+      <c r="K25" s="148"/>
+      <c r="L25" s="148"/>
+      <c r="M25" s="148"/>
+      <c r="N25" s="148"/>
+      <c r="O25" s="148"/>
+      <c r="P25" s="148"/>
+      <c r="Q25" s="147"/>
+      <c r="R25" s="147"/>
+      <c r="S25" s="147"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="149"/>
-      <c r="C26" s="144" t="s">
+      <c r="B26" s="150"/>
+      <c r="C26" s="145" t="s">
         <v>265</v>
       </c>
-      <c r="D26" s="153" t="s">
+      <c r="D26" s="154" t="s">
         <v>266</v>
       </c>
-      <c r="E26" s="153" t="s">
+      <c r="E26" s="154" t="s">
         <v>158</v>
       </c>
-      <c r="F26" s="153"/>
-      <c r="G26" s="153"/>
-      <c r="H26" s="147"/>
-      <c r="I26" s="147"/>
-      <c r="J26" s="147"/>
-      <c r="K26" s="147"/>
-      <c r="L26" s="147"/>
-      <c r="M26" s="146"/>
-      <c r="N26" s="146"/>
-      <c r="O26" s="146"/>
-      <c r="P26" s="146"/>
-      <c r="Q26" s="146"/>
-      <c r="R26" s="146"/>
-      <c r="S26" s="146"/>
+      <c r="F26" s="154"/>
+      <c r="G26" s="154"/>
+      <c r="H26" s="148"/>
+      <c r="I26" s="148"/>
+      <c r="J26" s="148"/>
+      <c r="K26" s="148"/>
+      <c r="L26" s="148"/>
+      <c r="M26" s="147"/>
+      <c r="N26" s="147"/>
+      <c r="O26" s="147"/>
+      <c r="P26" s="147"/>
+      <c r="Q26" s="147"/>
+      <c r="R26" s="147"/>
+      <c r="S26" s="147"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="149"/>
-      <c r="C27" s="159" t="s">
+      <c r="B27" s="150"/>
+      <c r="C27" s="160" t="s">
         <v>267</v>
       </c>
-      <c r="D27" s="160" t="s">
+      <c r="D27" s="161" t="s">
         <v>268</v>
       </c>
-      <c r="E27" s="160"/>
-      <c r="F27" s="160"/>
-      <c r="G27" s="160"/>
-      <c r="H27" s="146"/>
-      <c r="I27" s="146"/>
-      <c r="J27" s="146"/>
-      <c r="K27" s="146"/>
-      <c r="L27" s="146"/>
-      <c r="M27" s="146"/>
-      <c r="N27" s="146"/>
-      <c r="O27" s="146"/>
-      <c r="P27" s="146"/>
-      <c r="Q27" s="146"/>
-      <c r="R27" s="146"/>
-      <c r="S27" s="146"/>
+      <c r="E27" s="161"/>
+      <c r="F27" s="161"/>
+      <c r="G27" s="161"/>
+      <c r="H27" s="147"/>
+      <c r="I27" s="147"/>
+      <c r="J27" s="147"/>
+      <c r="K27" s="147"/>
+      <c r="L27" s="147"/>
+      <c r="M27" s="147"/>
+      <c r="N27" s="147"/>
+      <c r="O27" s="147"/>
+      <c r="P27" s="147"/>
+      <c r="Q27" s="147"/>
+      <c r="R27" s="147"/>
+      <c r="S27" s="147"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="148" t="n">
+      <c r="A28" s="149" t="n">
         <v>4</v>
       </c>
-      <c r="B28" s="149"/>
-      <c r="C28" s="161" t="s">
+      <c r="B28" s="150"/>
+      <c r="C28" s="162" t="s">
         <v>269</v>
       </c>
-      <c r="D28" s="160" t="s">
+      <c r="D28" s="161" t="s">
         <v>270</v>
       </c>
-      <c r="E28" s="160"/>
-      <c r="F28" s="160"/>
-      <c r="G28" s="160"/>
-      <c r="H28" s="146"/>
-      <c r="I28" s="146"/>
-      <c r="J28" s="146"/>
-      <c r="K28" s="146"/>
-      <c r="L28" s="146"/>
-      <c r="M28" s="146"/>
-      <c r="N28" s="146"/>
-      <c r="O28" s="146"/>
-      <c r="P28" s="146"/>
-      <c r="Q28" s="146"/>
-      <c r="R28" s="146"/>
-      <c r="S28" s="146"/>
+      <c r="E28" s="161"/>
+      <c r="F28" s="161"/>
+      <c r="G28" s="161"/>
+      <c r="H28" s="147"/>
+      <c r="I28" s="147"/>
+      <c r="J28" s="147"/>
+      <c r="K28" s="147"/>
+      <c r="L28" s="147"/>
+      <c r="M28" s="147"/>
+      <c r="N28" s="147"/>
+      <c r="O28" s="147"/>
+      <c r="P28" s="147"/>
+      <c r="Q28" s="147"/>
+      <c r="R28" s="147"/>
+      <c r="S28" s="147"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="149"/>
-      <c r="C29" s="161" t="s">
+      <c r="B29" s="150"/>
+      <c r="C29" s="162" t="s">
         <v>271</v>
       </c>
-      <c r="D29" s="160" t="s">
+      <c r="D29" s="161" t="s">
         <v>272</v>
       </c>
-      <c r="E29" s="160"/>
-      <c r="F29" s="160"/>
-      <c r="G29" s="160"/>
-      <c r="H29" s="146"/>
-      <c r="I29" s="146"/>
-      <c r="J29" s="146"/>
-      <c r="K29" s="146"/>
-      <c r="L29" s="146"/>
-      <c r="M29" s="146"/>
-      <c r="N29" s="146"/>
-      <c r="O29" s="146"/>
-      <c r="P29" s="146"/>
-      <c r="Q29" s="146"/>
-      <c r="R29" s="146"/>
-      <c r="S29" s="146"/>
+      <c r="E29" s="161"/>
+      <c r="F29" s="161"/>
+      <c r="G29" s="161"/>
+      <c r="H29" s="147"/>
+      <c r="I29" s="147"/>
+      <c r="J29" s="147"/>
+      <c r="K29" s="147"/>
+      <c r="L29" s="147"/>
+      <c r="M29" s="147"/>
+      <c r="N29" s="147"/>
+      <c r="O29" s="147"/>
+      <c r="P29" s="147"/>
+      <c r="Q29" s="147"/>
+      <c r="R29" s="147"/>
+      <c r="S29" s="147"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="149"/>
-      <c r="C30" s="161" t="s">
+      <c r="B30" s="150"/>
+      <c r="C30" s="162" t="s">
         <v>273</v>
       </c>
-      <c r="D30" s="160" t="s">
+      <c r="D30" s="161" t="s">
         <v>274</v>
       </c>
-      <c r="E30" s="160"/>
-      <c r="F30" s="160"/>
-      <c r="G30" s="160"/>
-      <c r="H30" s="146"/>
-      <c r="I30" s="146"/>
-      <c r="J30" s="146"/>
-      <c r="K30" s="146"/>
-      <c r="L30" s="146"/>
-      <c r="M30" s="146"/>
-      <c r="N30" s="146"/>
-      <c r="O30" s="146"/>
-      <c r="P30" s="146"/>
-      <c r="Q30" s="146"/>
-      <c r="R30" s="146"/>
-      <c r="S30" s="146"/>
+      <c r="E30" s="161"/>
+      <c r="F30" s="161"/>
+      <c r="G30" s="161"/>
+      <c r="H30" s="147"/>
+      <c r="I30" s="147"/>
+      <c r="J30" s="147"/>
+      <c r="K30" s="147"/>
+      <c r="L30" s="147"/>
+      <c r="M30" s="147"/>
+      <c r="N30" s="147"/>
+      <c r="O30" s="147"/>
+      <c r="P30" s="147"/>
+      <c r="Q30" s="147"/>
+      <c r="R30" s="147"/>
+      <c r="S30" s="147"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="149"/>
-      <c r="C31" s="161" t="s">
+      <c r="B31" s="150"/>
+      <c r="C31" s="162" t="s">
         <v>275</v>
       </c>
-      <c r="D31" s="160" t="s">
+      <c r="D31" s="161" t="s">
         <v>276</v>
       </c>
-      <c r="E31" s="160"/>
-      <c r="F31" s="160"/>
-      <c r="G31" s="160"/>
-      <c r="H31" s="146"/>
-      <c r="I31" s="146"/>
-      <c r="J31" s="146"/>
-      <c r="K31" s="146"/>
-      <c r="L31" s="146"/>
-      <c r="M31" s="146"/>
-      <c r="N31" s="146"/>
-      <c r="O31" s="146"/>
-      <c r="P31" s="146"/>
-      <c r="Q31" s="146"/>
-      <c r="R31" s="146"/>
-      <c r="S31" s="146"/>
+      <c r="E31" s="161"/>
+      <c r="F31" s="161"/>
+      <c r="G31" s="161"/>
+      <c r="H31" s="147"/>
+      <c r="I31" s="147"/>
+      <c r="J31" s="147"/>
+      <c r="K31" s="147"/>
+      <c r="L31" s="147"/>
+      <c r="M31" s="147"/>
+      <c r="N31" s="147"/>
+      <c r="O31" s="147"/>
+      <c r="P31" s="147"/>
+      <c r="Q31" s="147"/>
+      <c r="R31" s="147"/>
+      <c r="S31" s="147"/>
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="162"/>
-      <c r="C32" s="160" t="s">
+      <c r="B32" s="163"/>
+      <c r="C32" s="161" t="s">
         <v>277</v>
       </c>
-      <c r="D32" s="160" t="s">
+      <c r="D32" s="161" t="s">
         <v>278</v>
       </c>
-      <c r="E32" s="160"/>
-      <c r="F32" s="160"/>
-      <c r="G32" s="160"/>
-      <c r="H32" s="146"/>
-      <c r="I32" s="146"/>
-      <c r="J32" s="146"/>
-      <c r="K32" s="146"/>
-      <c r="L32" s="146"/>
-      <c r="M32" s="146"/>
-      <c r="N32" s="146"/>
-      <c r="O32" s="146"/>
-      <c r="P32" s="146"/>
-      <c r="Q32" s="146"/>
-      <c r="R32" s="146"/>
-      <c r="S32" s="146"/>
+      <c r="E32" s="161"/>
+      <c r="F32" s="161"/>
+      <c r="G32" s="161"/>
+      <c r="H32" s="147"/>
+      <c r="I32" s="147"/>
+      <c r="J32" s="147"/>
+      <c r="K32" s="147"/>
+      <c r="L32" s="147"/>
+      <c r="M32" s="147"/>
+      <c r="N32" s="147"/>
+      <c r="O32" s="147"/>
+      <c r="P32" s="147"/>
+      <c r="Q32" s="147"/>
+      <c r="R32" s="147"/>
+      <c r="S32" s="147"/>
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C34" s="139" t="s">
+      <c r="C34" s="140" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C35" s="139" t="s">
+      <c r="C35" s="140" t="s">
         <v>279</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill remaining budget 2027 rows from grouped and salestype sources
Fills all 31 matchable category rows (K/L/N/O/P/Q, annualized 2026)
in the "שנים" sheet. Pharmacies and Meuhedet rows combine money-only
totals (Amount 2025/NEW/2026-annualized) summed across the grouped
and salestype sources per the dual-reporting-system reconciliation,
leaving their quantity columns blank. Notes 3 budget rows with no
matching source category (REMEDICARE, Quadrifoglio Medical Romania,
Young In Healthcare Korea) and 3 source categories with no matching
budget row (0Pharmim, Chemipal, Shoe Stores) for follow-up.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-09-20-budget-2027.xlsx
+++ b/kirill/outputs/2026-09-20-budget-2027.xlsx
@@ -11066,12 +11066,24 @@
       <c r="I5" s="96" t="n">
         <v>1037274.565</v>
       </c>
-      <c r="K5" s="100"/>
-      <c r="L5" s="100"/>
-      <c r="N5" s="100"/>
-      <c r="O5" s="100"/>
-      <c r="P5" s="100"/>
-      <c r="Q5" s="100"/>
+      <c r="K5" s="97" t="n">
+        <v>27268</v>
+      </c>
+      <c r="L5" s="97" t="n">
+        <v>889501.1</v>
+      </c>
+      <c r="N5" s="97" t="n">
+        <v>8</v>
+      </c>
+      <c r="O5" s="97" t="n">
+        <v>918.4</v>
+      </c>
+      <c r="P5" s="97" t="n">
+        <v>24137.6842105263</v>
+      </c>
+      <c r="Q5" s="97" t="n">
+        <v>854230.484210526</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="99" t="n">
@@ -11102,11 +11114,17 @@
         <v>2118523.978</v>
       </c>
       <c r="K6" s="100"/>
-      <c r="L6" s="100"/>
+      <c r="L6" s="97" t="n">
+        <v>2120059.06</v>
+      </c>
       <c r="N6" s="100"/>
-      <c r="O6" s="100"/>
+      <c r="O6" s="97" t="n">
+        <v>63207.99</v>
+      </c>
       <c r="P6" s="100"/>
-      <c r="Q6" s="100"/>
+      <c r="Q6" s="97" t="n">
+        <v>1774351.41473685</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="99" t="n">
@@ -11136,12 +11154,24 @@
       <c r="I7" s="96" t="n">
         <v>3722410.85</v>
       </c>
-      <c r="K7" s="100"/>
-      <c r="L7" s="100"/>
-      <c r="N7" s="100"/>
-      <c r="O7" s="100"/>
-      <c r="P7" s="100"/>
-      <c r="Q7" s="100"/>
+      <c r="K7" s="97" t="n">
+        <v>152395</v>
+      </c>
+      <c r="L7" s="97" t="n">
+        <v>3809616.42</v>
+      </c>
+      <c r="N7" s="97" t="n">
+        <v>-2</v>
+      </c>
+      <c r="O7" s="97" t="n">
+        <v>-1176</v>
+      </c>
+      <c r="P7" s="97" t="n">
+        <v>139120.421052632</v>
+      </c>
+      <c r="Q7" s="97" t="n">
+        <v>3245877.53684211</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="99" t="n">
@@ -11172,11 +11202,17 @@
         <v>943097.611</v>
       </c>
       <c r="K8" s="96"/>
-      <c r="L8" s="96"/>
+      <c r="L8" s="97" t="n">
+        <v>860680.72</v>
+      </c>
       <c r="N8" s="96"/>
-      <c r="O8" s="96"/>
+      <c r="O8" s="97" t="n">
+        <v>308751.05</v>
+      </c>
       <c r="P8" s="96"/>
-      <c r="Q8" s="96"/>
+      <c r="Q8" s="97" t="n">
+        <v>624255.688421052</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="99" t="n">
@@ -11206,12 +11242,24 @@
       <c r="I9" s="96" t="n">
         <v>1075277.57</v>
       </c>
-      <c r="K9" s="100"/>
-      <c r="L9" s="100"/>
-      <c r="N9" s="100"/>
-      <c r="O9" s="100"/>
-      <c r="P9" s="100"/>
-      <c r="Q9" s="100"/>
+      <c r="K9" s="97" t="n">
+        <v>11637</v>
+      </c>
+      <c r="L9" s="97" t="n">
+        <v>850045.24</v>
+      </c>
+      <c r="N9" s="97" t="n">
+        <v>728</v>
+      </c>
+      <c r="O9" s="97" t="n">
+        <v>56220.09</v>
+      </c>
+      <c r="P9" s="97" t="n">
+        <v>9871.57894736842</v>
+      </c>
+      <c r="Q9" s="97" t="n">
+        <v>818053.907368421</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="101" t="n">
@@ -11241,12 +11289,24 @@
       <c r="I10" s="96" t="n">
         <v>151235.08</v>
       </c>
-      <c r="K10" s="100"/>
-      <c r="L10" s="100"/>
-      <c r="N10" s="100"/>
-      <c r="O10" s="100"/>
-      <c r="P10" s="100"/>
-      <c r="Q10" s="100"/>
+      <c r="K10" s="97" t="n">
+        <v>3679</v>
+      </c>
+      <c r="L10" s="97" t="n">
+        <v>185250.51</v>
+      </c>
+      <c r="N10" s="97" t="n">
+        <v>253</v>
+      </c>
+      <c r="O10" s="97" t="n">
+        <v>13716.33</v>
+      </c>
+      <c r="P10" s="97" t="n">
+        <v>1740.63157894737</v>
+      </c>
+      <c r="Q10" s="97" t="n">
+        <v>98772.012631579</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="99" t="n">
@@ -11276,12 +11336,24 @@
       <c r="I11" s="96" t="n">
         <v>94015.41</v>
       </c>
-      <c r="K11" s="100"/>
-      <c r="L11" s="100"/>
-      <c r="N11" s="100"/>
-      <c r="O11" s="100"/>
-      <c r="P11" s="100"/>
-      <c r="Q11" s="100"/>
+      <c r="K11" s="97" t="n">
+        <v>1208</v>
+      </c>
+      <c r="L11" s="97" t="n">
+        <v>58306.79</v>
+      </c>
+      <c r="N11" s="97" t="n">
+        <v>244</v>
+      </c>
+      <c r="O11" s="97" t="n">
+        <v>18033.75</v>
+      </c>
+      <c r="P11" s="97" t="n">
+        <v>833.684210526316</v>
+      </c>
+      <c r="Q11" s="97" t="n">
+        <v>58745.8736842105</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="99" t="n">
@@ -11311,12 +11383,24 @@
       <c r="I12" s="96" t="n">
         <v>33576.15</v>
       </c>
-      <c r="K12" s="100"/>
-      <c r="L12" s="100"/>
-      <c r="N12" s="100"/>
-      <c r="O12" s="100"/>
-      <c r="P12" s="100"/>
-      <c r="Q12" s="100"/>
+      <c r="K12" s="97" t="n">
+        <v>114</v>
+      </c>
+      <c r="L12" s="97" t="n">
+        <v>4145.68</v>
+      </c>
+      <c r="N12" s="97" t="n">
+        <v>18</v>
+      </c>
+      <c r="O12" s="97" t="n">
+        <v>1012.72</v>
+      </c>
+      <c r="P12" s="97" t="n">
+        <v>122.526315789474</v>
+      </c>
+      <c r="Q12" s="97" t="n">
+        <v>5437.92</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="99" t="n">
@@ -11346,12 +11430,24 @@
       <c r="I13" s="96" t="n">
         <v>31896.82</v>
       </c>
-      <c r="K13" s="100"/>
-      <c r="L13" s="100"/>
-      <c r="N13" s="100"/>
-      <c r="O13" s="100"/>
-      <c r="P13" s="100"/>
-      <c r="Q13" s="100"/>
+      <c r="K13" s="97" t="n">
+        <v>16</v>
+      </c>
+      <c r="L13" s="97" t="n">
+        <v>514.2</v>
+      </c>
+      <c r="N13" s="97" t="n">
+        <v>59</v>
+      </c>
+      <c r="O13" s="97" t="n">
+        <v>1896.82</v>
+      </c>
+      <c r="P13" s="97" t="n">
+        <v>74.5263157894737</v>
+      </c>
+      <c r="Q13" s="97" t="n">
+        <v>2395.98315789474</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="99" t="n">
@@ -11381,12 +11477,24 @@
       <c r="I14" s="96" t="n">
         <v>37748.72</v>
       </c>
-      <c r="K14" s="100"/>
-      <c r="L14" s="100"/>
-      <c r="N14" s="100"/>
-      <c r="O14" s="100"/>
-      <c r="P14" s="100"/>
-      <c r="Q14" s="100"/>
+      <c r="K14" s="97" t="n">
+        <v>286</v>
+      </c>
+      <c r="L14" s="97" t="n">
+        <v>13532.23</v>
+      </c>
+      <c r="N14" s="97" t="n">
+        <v>41</v>
+      </c>
+      <c r="O14" s="97" t="n">
+        <v>4381.47</v>
+      </c>
+      <c r="P14" s="97" t="n">
+        <v>261.473684210526</v>
+      </c>
+      <c r="Q14" s="97" t="n">
+        <v>14829.2589473684</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="99" t="n">
@@ -11416,12 +11524,24 @@
       <c r="I15" s="96" t="n">
         <v>239111.1</v>
       </c>
-      <c r="K15" s="100"/>
-      <c r="L15" s="100"/>
-      <c r="N15" s="100"/>
-      <c r="O15" s="100"/>
-      <c r="P15" s="100"/>
-      <c r="Q15" s="100"/>
+      <c r="K15" s="97" t="n">
+        <v>1673</v>
+      </c>
+      <c r="L15" s="97" t="n">
+        <v>98528.23</v>
+      </c>
+      <c r="N15" s="97" t="n">
+        <v>322</v>
+      </c>
+      <c r="O15" s="97" t="n">
+        <v>27429.03</v>
+      </c>
+      <c r="P15" s="97" t="n">
+        <v>1917.47368421053</v>
+      </c>
+      <c r="Q15" s="97" t="n">
+        <v>143175.309473684</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="102"/>
@@ -11451,21 +11571,21 @@
       </c>
       <c r="K16" s="103" t="n">
         <f aca="false">SUM(K3:K15)</f>
-        <v>294897</v>
+        <v>493173</v>
       </c>
       <c r="L16" s="103" t="n">
         <f aca="false">SUM(L3:L15)</f>
-        <v>8397877.35</v>
+        <v>17288057.53</v>
       </c>
       <c r="N16" s="103" t="n">
         <f aca="false">SUM(N3:N15)</f>
-        <v>1952</v>
+        <v>3623</v>
       </c>
       <c r="O16" s="103"/>
       <c r="P16" s="103"/>
       <c r="Q16" s="103" t="n">
         <f aca="false">SUM(Q3:Q15)</f>
-        <v>7061493.66315789</v>
+        <v>14701619.0526316</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11543,12 +11663,24 @@
       <c r="I18" s="96" t="n">
         <v>39807.02</v>
       </c>
-      <c r="K18" s="100"/>
-      <c r="L18" s="100"/>
-      <c r="N18" s="100"/>
-      <c r="O18" s="100"/>
-      <c r="P18" s="100"/>
-      <c r="Q18" s="100"/>
+      <c r="K18" s="97" t="n">
+        <v>415</v>
+      </c>
+      <c r="L18" s="97" t="n">
+        <v>27325.74</v>
+      </c>
+      <c r="N18" s="97" t="n">
+        <v>12</v>
+      </c>
+      <c r="O18" s="97" t="n">
+        <v>1716.98</v>
+      </c>
+      <c r="P18" s="97" t="n">
+        <v>252.631578947368</v>
+      </c>
+      <c r="Q18" s="97" t="n">
+        <v>16463.3178947368</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="101"/>
@@ -11578,21 +11710,21 @@
       </c>
       <c r="K19" s="103" t="n">
         <f aca="false">K16+K17+K18</f>
-        <v>315367</v>
+        <v>514058</v>
       </c>
       <c r="L19" s="103" t="n">
         <f aca="false">L16+L17+L18</f>
-        <v>10055198.11</v>
+        <v>18972704.03</v>
       </c>
       <c r="N19" s="103" t="n">
         <f aca="false">N16+N17+N18</f>
-        <v>4327</v>
+        <v>6010</v>
       </c>
       <c r="O19" s="103"/>
       <c r="P19" s="103"/>
       <c r="Q19" s="103" t="n">
         <f aca="false">Q16+Q17+Q18</f>
-        <v>11099140.1431579</v>
+        <v>18755728.8505263</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11623,12 +11755,24 @@
       <c r="I20" s="96" t="n">
         <v>3098024.51</v>
       </c>
-      <c r="K20" s="100"/>
-      <c r="L20" s="100"/>
-      <c r="N20" s="100"/>
-      <c r="O20" s="100"/>
-      <c r="P20" s="100"/>
-      <c r="Q20" s="100"/>
+      <c r="K20" s="97" t="n">
+        <v>27158</v>
+      </c>
+      <c r="L20" s="97" t="n">
+        <v>2705391.22</v>
+      </c>
+      <c r="N20" s="97" t="n">
+        <v>47</v>
+      </c>
+      <c r="O20" s="97" t="n">
+        <v>3274.06</v>
+      </c>
+      <c r="P20" s="97" t="n">
+        <v>23757.4736842105</v>
+      </c>
+      <c r="Q20" s="97" t="n">
+        <v>2062598.93052632</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="101" t="n">
@@ -11658,12 +11802,24 @@
       <c r="I21" s="96" t="n">
         <v>922081.02</v>
       </c>
-      <c r="K21" s="100"/>
-      <c r="L21" s="100"/>
-      <c r="N21" s="100"/>
-      <c r="O21" s="100"/>
-      <c r="P21" s="100"/>
-      <c r="Q21" s="100"/>
+      <c r="K21" s="97" t="n">
+        <v>48363</v>
+      </c>
+      <c r="L21" s="97" t="n">
+        <v>902537.64</v>
+      </c>
+      <c r="N21" s="97" t="n">
+        <v>250</v>
+      </c>
+      <c r="O21" s="97" t="n">
+        <v>11540.57</v>
+      </c>
+      <c r="P21" s="97" t="n">
+        <v>35605.8947368421</v>
+      </c>
+      <c r="Q21" s="97" t="n">
+        <v>598967.482105263</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="101" t="n">
@@ -11693,12 +11849,24 @@
       <c r="I22" s="96" t="n">
         <v>613276.52</v>
       </c>
-      <c r="K22" s="100"/>
-      <c r="L22" s="100"/>
-      <c r="N22" s="100"/>
-      <c r="O22" s="100"/>
-      <c r="P22" s="100"/>
-      <c r="Q22" s="100"/>
+      <c r="K22" s="97" t="n">
+        <v>6959</v>
+      </c>
+      <c r="L22" s="97" t="n">
+        <v>405920.85</v>
+      </c>
+      <c r="N22" s="97" t="n">
+        <v>131</v>
+      </c>
+      <c r="O22" s="97" t="n">
+        <v>4054.38</v>
+      </c>
+      <c r="P22" s="97" t="n">
+        <v>8513.68421052632</v>
+      </c>
+      <c r="Q22" s="97" t="n">
+        <v>434858.64</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="101" t="n">
@@ -11728,12 +11896,24 @@
       <c r="I23" s="96" t="n">
         <v>457053.13</v>
       </c>
-      <c r="K23" s="100"/>
-      <c r="L23" s="100"/>
-      <c r="N23" s="100"/>
-      <c r="O23" s="100"/>
-      <c r="P23" s="100"/>
-      <c r="Q23" s="100"/>
+      <c r="K23" s="97" t="n">
+        <v>21177</v>
+      </c>
+      <c r="L23" s="97" t="n">
+        <v>414072.64</v>
+      </c>
+      <c r="N23" s="97" t="n">
+        <v>154</v>
+      </c>
+      <c r="O23" s="97" t="n">
+        <v>3246.9</v>
+      </c>
+      <c r="P23" s="97" t="n">
+        <v>22898.5263157895</v>
+      </c>
+      <c r="Q23" s="97" t="n">
+        <v>387859.162105263</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="101" t="n">
@@ -11763,12 +11943,24 @@
       <c r="I24" s="96" t="n">
         <v>131678.59</v>
       </c>
-      <c r="K24" s="100"/>
-      <c r="L24" s="100"/>
-      <c r="N24" s="100"/>
-      <c r="O24" s="100"/>
-      <c r="P24" s="100"/>
-      <c r="Q24" s="100"/>
+      <c r="K24" s="97" t="n">
+        <v>12986</v>
+      </c>
+      <c r="L24" s="97" t="n">
+        <v>122339</v>
+      </c>
+      <c r="N24" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="97" t="n">
+        <v>16302.3157894737</v>
+      </c>
+      <c r="Q24" s="97" t="n">
+        <v>121427.141052632</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="101" t="n">
@@ -11798,12 +11990,24 @@
       <c r="I25" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="100"/>
-      <c r="L25" s="100"/>
-      <c r="N25" s="100"/>
-      <c r="O25" s="100"/>
-      <c r="P25" s="100"/>
-      <c r="Q25" s="100"/>
+      <c r="K25" s="97" t="n">
+        <v>1817</v>
+      </c>
+      <c r="L25" s="97" t="n">
+        <v>52899.82</v>
+      </c>
+      <c r="N25" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="101" t="n">
@@ -11880,12 +12084,24 @@
       <c r="I27" s="96" t="n">
         <v>100694.01</v>
       </c>
-      <c r="K27" s="100"/>
-      <c r="L27" s="100"/>
-      <c r="N27" s="100"/>
-      <c r="O27" s="100"/>
-      <c r="P27" s="100"/>
-      <c r="Q27" s="100"/>
+      <c r="K27" s="97" t="n">
+        <v>3507</v>
+      </c>
+      <c r="L27" s="97" t="n">
+        <v>86855.65</v>
+      </c>
+      <c r="N27" s="97" t="n">
+        <v>754</v>
+      </c>
+      <c r="O27" s="97" t="n">
+        <v>27727.77</v>
+      </c>
+      <c r="P27" s="97" t="n">
+        <v>2952</v>
+      </c>
+      <c r="Q27" s="97" t="n">
+        <v>76373.5452631579</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="101" t="n">
@@ -11915,12 +12131,24 @@
       <c r="I28" s="96" t="n">
         <v>250000</v>
       </c>
-      <c r="K28" s="100"/>
-      <c r="L28" s="100"/>
-      <c r="N28" s="100"/>
-      <c r="O28" s="100"/>
-      <c r="P28" s="100"/>
-      <c r="Q28" s="100"/>
+      <c r="K28" s="97" t="n">
+        <v>6687</v>
+      </c>
+      <c r="L28" s="97" t="n">
+        <v>256772.1</v>
+      </c>
+      <c r="N28" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="101" t="n">
@@ -11950,12 +12178,24 @@
       <c r="I29" s="96" t="n">
         <v>378207.09</v>
       </c>
-      <c r="K29" s="100"/>
-      <c r="L29" s="100"/>
-      <c r="N29" s="100"/>
-      <c r="O29" s="100"/>
-      <c r="P29" s="100"/>
-      <c r="Q29" s="100"/>
+      <c r="K29" s="97" t="n">
+        <v>13479</v>
+      </c>
+      <c r="L29" s="97" t="n">
+        <v>407234.61</v>
+      </c>
+      <c r="N29" s="97" t="n">
+        <v>147</v>
+      </c>
+      <c r="O29" s="97" t="n">
+        <v>6167.14</v>
+      </c>
+      <c r="P29" s="97" t="n">
+        <v>12256.4210526316</v>
+      </c>
+      <c r="Q29" s="97" t="n">
+        <v>380002.345263158</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="101" t="n">
@@ -11985,12 +12225,24 @@
       <c r="I30" s="96" t="n">
         <v>73116.44</v>
       </c>
-      <c r="K30" s="100"/>
-      <c r="L30" s="100"/>
-      <c r="N30" s="100"/>
-      <c r="O30" s="100"/>
-      <c r="P30" s="100"/>
-      <c r="Q30" s="100"/>
+      <c r="K30" s="97" t="n">
+        <v>2672</v>
+      </c>
+      <c r="L30" s="97" t="n">
+        <v>64554.59</v>
+      </c>
+      <c r="N30" s="97" t="n">
+        <v>360</v>
+      </c>
+      <c r="O30" s="97" t="n">
+        <v>16342.42</v>
+      </c>
+      <c r="P30" s="97" t="n">
+        <v>1914.94736842105</v>
+      </c>
+      <c r="Q30" s="97" t="n">
+        <v>54462.8715789474</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="101" t="n">
@@ -12020,12 +12272,24 @@
       <c r="I31" s="96" t="n">
         <v>42809.5</v>
       </c>
-      <c r="K31" s="100"/>
-      <c r="L31" s="100"/>
-      <c r="N31" s="100"/>
-      <c r="O31" s="100"/>
-      <c r="P31" s="100"/>
-      <c r="Q31" s="100"/>
+      <c r="K31" s="97" t="n">
+        <v>2980</v>
+      </c>
+      <c r="L31" s="97" t="n">
+        <v>60908.2</v>
+      </c>
+      <c r="N31" s="97" t="n">
+        <v>260</v>
+      </c>
+      <c r="O31" s="97" t="n">
+        <v>5860.29</v>
+      </c>
+      <c r="P31" s="97" t="n">
+        <v>2058.94736842105</v>
+      </c>
+      <c r="Q31" s="97" t="n">
+        <v>41437.3768421053</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="101" t="n">
@@ -12055,12 +12319,24 @@
       <c r="I32" s="96" t="n">
         <v>17500</v>
       </c>
-      <c r="K32" s="100"/>
-      <c r="L32" s="100"/>
-      <c r="N32" s="100"/>
-      <c r="O32" s="100"/>
-      <c r="P32" s="100"/>
-      <c r="Q32" s="100"/>
+      <c r="K32" s="97" t="n">
+        <v>3060</v>
+      </c>
+      <c r="L32" s="97" t="n">
+        <v>81786.57</v>
+      </c>
+      <c r="N32" s="97" t="n">
+        <v>5</v>
+      </c>
+      <c r="O32" s="97" t="n">
+        <v>86.54</v>
+      </c>
+      <c r="P32" s="97" t="n">
+        <v>851.368421052631</v>
+      </c>
+      <c r="Q32" s="97" t="n">
+        <v>12678.5052631579</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="101"/>
@@ -12119,12 +12395,24 @@
       <c r="I34" s="96" t="n">
         <v>38792.66</v>
       </c>
-      <c r="K34" s="100"/>
-      <c r="L34" s="100"/>
-      <c r="N34" s="100"/>
-      <c r="O34" s="100"/>
-      <c r="P34" s="100"/>
-      <c r="Q34" s="100"/>
+      <c r="K34" s="97" t="n">
+        <v>1359</v>
+      </c>
+      <c r="L34" s="97" t="n">
+        <v>39713.57</v>
+      </c>
+      <c r="N34" s="97" t="n">
+        <v>56</v>
+      </c>
+      <c r="O34" s="97" t="n">
+        <v>1430.29</v>
+      </c>
+      <c r="P34" s="97" t="n">
+        <v>1935.15789473684</v>
+      </c>
+      <c r="Q34" s="97" t="n">
+        <v>46917.1452631579</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="101" t="n">
@@ -12154,12 +12442,24 @@
       <c r="I35" s="96" t="n">
         <v>25000</v>
       </c>
-      <c r="K35" s="100"/>
-      <c r="L35" s="100"/>
-      <c r="N35" s="100"/>
-      <c r="O35" s="100"/>
-      <c r="P35" s="100"/>
-      <c r="Q35" s="100"/>
+      <c r="K35" s="97" t="n">
+        <v>1737</v>
+      </c>
+      <c r="L35" s="97" t="n">
+        <v>53863.18</v>
+      </c>
+      <c r="N35" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" s="97" t="n">
+        <v>1235.36842105263</v>
+      </c>
+      <c r="Q35" s="97" t="n">
+        <v>32975.6463157895</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="101"/>
@@ -12257,12 +12557,24 @@
       <c r="I38" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="K38" s="100"/>
-      <c r="L38" s="100"/>
-      <c r="N38" s="100"/>
-      <c r="O38" s="100"/>
-      <c r="P38" s="100"/>
-      <c r="Q38" s="100"/>
+      <c r="K38" s="97" t="n">
+        <v>24</v>
+      </c>
+      <c r="L38" s="97" t="n">
+        <v>248.59</v>
+      </c>
+      <c r="N38" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="101" t="n">
@@ -12371,21 +12683,21 @@
       </c>
       <c r="K42" s="104" t="n">
         <f aca="false">SUM(K20:K41)</f>
-        <v>18268</v>
+        <v>172233</v>
       </c>
       <c r="L42" s="104" t="n">
         <f aca="false">SUM(L20:L41)</f>
-        <v>319558.55</v>
+        <v>5974656.78</v>
       </c>
       <c r="N42" s="104" t="n">
         <f aca="false">SUM(N20:N41)</f>
-        <v>991</v>
+        <v>3155</v>
       </c>
       <c r="O42" s="104"/>
       <c r="P42" s="104"/>
       <c r="Q42" s="104" t="n">
         <f aca="false">SUM(Q20:Q41)</f>
-        <v>461754</v>
+        <v>4712312.79157895</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12416,21 +12728,21 @@
       </c>
       <c r="K43" s="105" t="n">
         <f aca="false">K42+K19</f>
-        <v>333635</v>
+        <v>686291</v>
       </c>
       <c r="L43" s="105" t="n">
         <f aca="false">L42+L19</f>
-        <v>10374756.66</v>
+        <v>24947360.81</v>
       </c>
       <c r="N43" s="105" t="n">
         <f aca="false">N42+N19</f>
-        <v>5318</v>
+        <v>9165</v>
       </c>
       <c r="O43" s="105"/>
       <c r="P43" s="105"/>
       <c r="Q43" s="105" t="n">
         <f aca="false">Q42+Q19</f>
-        <v>11560894.1431579</v>
+        <v>23468041.6421053</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12460,21 +12772,21 @@
       </c>
       <c r="K44" s="107" t="n">
         <f aca="false">IFERROR(K42/K43,"")</f>
-        <v>0.0547544472252611</v>
+        <v>0.25096205545461</v>
       </c>
       <c r="L44" s="107" t="n">
         <f aca="false">IFERROR(L42/L43,"")</f>
-        <v>0.0308015465299598</v>
+        <v>0.239490534710393</v>
       </c>
       <c r="N44" s="107" t="n">
         <f aca="false">IFERROR(N42/N43,"")</f>
-        <v>0.186348251222264</v>
+        <v>0.344244408074195</v>
       </c>
       <c r="O44" s="107"/>
       <c r="P44" s="107"/>
       <c r="Q44" s="107" t="n">
         <f aca="false">IFERROR(Q42/Q43,"")</f>
-        <v>0.0399410282874427</v>
+        <v>0.20079701849192</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12519,7 +12831,7 @@
       </c>
       <c r="K47" s="108" t="n">
         <f aca="false">K16</f>
-        <v>294897</v>
+        <v>493173</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12545,7 +12857,7 @@
       </c>
       <c r="K48" s="108" t="n">
         <f aca="false">K17+K18</f>
-        <v>20470</v>
+        <v>20885</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12571,7 +12883,7 @@
       </c>
       <c r="K49" s="110" t="n">
         <f aca="false">SUM(K47:K48)</f>
-        <v>315367</v>
+        <v>514058</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12597,7 +12909,7 @@
       </c>
       <c r="K51" s="108" t="n">
         <f aca="false">K20</f>
-        <v>0</v>
+        <v>27158</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12623,7 +12935,7 @@
       </c>
       <c r="K52" s="108" t="n">
         <f aca="false">SUM(K21:K41)</f>
-        <v>18268</v>
+        <v>145075</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12649,7 +12961,7 @@
       </c>
       <c r="K53" s="105" t="n">
         <f aca="false">SUM(K49:K52)</f>
-        <v>333635</v>
+        <v>686291</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>